<commit_message>
Rate check: add more Pakistani-store sources, update revised quotation
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
@@ -739,7 +739,7 @@
     <t xml:space="preserve">FULL BODY HARNESS BELT</t>
   </si>
   <si>
-    <t xml:space="preserve">Karam</t>
+    <t xml:space="preserve">Toho (Taiwan)</t>
   </si>
   <si>
     <t xml:space="preserve">ANGLE GRINDER 9" BOSCH PRO STONE BONDED CU</t>
@@ -1325,11 +1325,11 @@
         <v>6</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1105</v>
+        <v>1150</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">D10*E10</f>
-        <v>6630</v>
+        <v>6900</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1451,11 +1451,11 @@
         <v>3</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>8620</v>
+        <v>8630</v>
       </c>
       <c r="F16" s="5" t="n">
         <f aca="false">D16*E16</f>
-        <v>25860</v>
+        <v>25890</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1766,11 +1766,11 @@
         <v>4</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>8620</v>
+        <v>8630</v>
       </c>
       <c r="F31" s="5" t="n">
         <f aca="false">D31*E31</f>
-        <v>34480</v>
+        <v>34520</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1787,11 +1787,11 @@
         <v>3</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>8620</v>
+        <v>8630</v>
       </c>
       <c r="F32" s="5" t="n">
         <f aca="false">D32*E32</f>
-        <v>25860</v>
+        <v>25890</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2102,11 +2102,11 @@
         <v>4</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>2640</v>
+        <v>2300</v>
       </c>
       <c r="F47" s="5" t="n">
         <f aca="false">D47*E47</f>
-        <v>10560</v>
+        <v>9200</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2123,11 +2123,11 @@
         <v>4</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>2640</v>
+        <v>2300</v>
       </c>
       <c r="F48" s="5" t="n">
         <f aca="false">D48*E48</f>
-        <v>10560</v>
+        <v>9200</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2438,11 +2438,11 @@
         <v>2</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>8620</v>
+        <v>8630</v>
       </c>
       <c r="F63" s="5" t="n">
         <f aca="false">D63*E63</f>
-        <v>17240</v>
+        <v>17260</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2501,11 +2501,11 @@
         <v>3</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>2070</v>
+        <v>1840</v>
       </c>
       <c r="F66" s="5" t="n">
         <f aca="false">D66*E66</f>
-        <v>6210</v>
+        <v>5520</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2522,11 +2522,11 @@
         <v>3</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>2070</v>
+        <v>1840</v>
       </c>
       <c r="F67" s="5" t="n">
         <f aca="false">D67*E67</f>
-        <v>6210</v>
+        <v>5520</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2942,11 +2942,11 @@
         <v>1</v>
       </c>
       <c r="E87" s="5" t="n">
-        <v>20120</v>
+        <v>20130</v>
       </c>
       <c r="F87" s="5" t="n">
         <f aca="false">D87*E87</f>
-        <v>20120</v>
+        <v>20130</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3236,11 +3236,11 @@
         <v>3</v>
       </c>
       <c r="E101" s="5" t="n">
-        <v>8620</v>
+        <v>8630</v>
       </c>
       <c r="F101" s="5" t="n">
         <f aca="false">D101*E101</f>
-        <v>25860</v>
+        <v>25890</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3866,11 +3866,11 @@
         <v>2</v>
       </c>
       <c r="E131" s="5" t="n">
-        <v>8050</v>
+        <v>7800</v>
       </c>
       <c r="F131" s="5" t="n">
         <f aca="false">D131*E131</f>
-        <v>16100</v>
+        <v>15600</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3971,11 +3971,11 @@
         <v>500</v>
       </c>
       <c r="E136" s="5" t="n">
-        <v>140</v>
+        <v>310</v>
       </c>
       <c r="F136" s="5" t="n">
         <f aca="false">D136*E136</f>
-        <v>70000</v>
+        <v>155000</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4286,11 +4286,11 @@
         <v>24</v>
       </c>
       <c r="E151" s="5" t="n">
-        <v>1105</v>
+        <v>1150</v>
       </c>
       <c r="F151" s="5" t="n">
         <f aca="false">D151*E151</f>
-        <v>26520</v>
+        <v>27600</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4496,11 +4496,11 @@
         <v>40</v>
       </c>
       <c r="E161" s="5" t="n">
-        <v>1260</v>
+        <v>1270</v>
       </c>
       <c r="F161" s="5" t="n">
         <f aca="false">D161*E161</f>
-        <v>50400</v>
+        <v>50800</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4517,11 +4517,11 @@
         <v>40</v>
       </c>
       <c r="E162" s="5" t="n">
-        <v>1260</v>
+        <v>1270</v>
       </c>
       <c r="F162" s="5" t="n">
         <f aca="false">D162*E162</f>
-        <v>50400</v>
+        <v>50800</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4769,11 +4769,11 @@
         <v>3</v>
       </c>
       <c r="E174" s="5" t="n">
-        <v>4940</v>
+        <v>4950</v>
       </c>
       <c r="F174" s="5" t="n">
         <f aca="false">D174*E174</f>
-        <v>14820</v>
+        <v>14850</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5000,11 +5000,11 @@
         <v>1</v>
       </c>
       <c r="E185" s="5" t="n">
-        <v>10800</v>
+        <v>7430</v>
       </c>
       <c r="F185" s="5" t="n">
         <f aca="false">D185*E185</f>
-        <v>10800</v>
+        <v>7430</v>
       </c>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5021,11 +5021,11 @@
         <v>1</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>12820</v>
+        <v>8780</v>
       </c>
       <c r="F186" s="5" t="n">
         <f aca="false">D186*E186</f>
-        <v>12820</v>
+        <v>8780</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5042,11 +5042,11 @@
         <v>1</v>
       </c>
       <c r="E187" s="5" t="n">
-        <v>19500</v>
+        <v>9720</v>
       </c>
       <c r="F187" s="5" t="n">
         <f aca="false">D187*E187</f>
-        <v>19500</v>
+        <v>9720</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5063,11 +5063,11 @@
         <v>1</v>
       </c>
       <c r="E188" s="5" t="n">
-        <v>20800</v>
+        <v>10530</v>
       </c>
       <c r="F188" s="5" t="n">
         <f aca="false">D188*E188</f>
-        <v>20800</v>
+        <v>10530</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5084,11 +5084,11 @@
         <v>1</v>
       </c>
       <c r="E189" s="5" t="n">
-        <v>22750</v>
+        <v>13230</v>
       </c>
       <c r="F189" s="5" t="n">
         <f aca="false">D189*E189</f>
-        <v>22750</v>
+        <v>13230</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5462,11 +5462,11 @@
         <v>1</v>
       </c>
       <c r="E207" s="5" t="n">
-        <v>2180</v>
+        <v>2190</v>
       </c>
       <c r="F207" s="5" t="n">
         <f aca="false">D207*E207</f>
-        <v>2180</v>
+        <v>2190</v>
       </c>
     </row>
     <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5588,11 +5588,11 @@
         <v>24</v>
       </c>
       <c r="E213" s="5" t="n">
-        <v>2180</v>
+        <v>2190</v>
       </c>
       <c r="F213" s="5" t="n">
         <f aca="false">D213*E213</f>
-        <v>52320</v>
+        <v>52560</v>
       </c>
     </row>
     <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5819,11 +5819,11 @@
         <v>6</v>
       </c>
       <c r="E224" s="5" t="n">
-        <v>10350</v>
+        <v>8970</v>
       </c>
       <c r="F224" s="5" t="n">
         <f aca="false">D224*E224</f>
-        <v>62100</v>
+        <v>53820</v>
       </c>
     </row>
     <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5874,7 +5874,7 @@
       </c>
       <c r="F227" s="7" t="n">
         <f aca="false">SUM(F5:F226)</f>
-        <v>13935976</v>
+        <v>13973706</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revised quotation: round rates half-up to match the rate check sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
@@ -1619,11 +1619,11 @@
         <v>3</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1490</v>
+        <v>1500</v>
       </c>
       <c r="F24" s="5" t="n">
         <f aca="false">D24*E24</f>
-        <v>4470</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1640,11 +1640,11 @@
         <v>3</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>1950</v>
+        <v>1960</v>
       </c>
       <c r="F25" s="5" t="n">
         <f aca="false">D25*E25</f>
-        <v>5850</v>
+        <v>5880</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1682,11 +1682,11 @@
         <v>4</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>6320</v>
+        <v>6330</v>
       </c>
       <c r="F27" s="5" t="n">
         <f aca="false">D27*E27</f>
-        <v>25280</v>
+        <v>25320</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1703,11 +1703,11 @@
         <v>4</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>6320</v>
+        <v>6330</v>
       </c>
       <c r="F28" s="5" t="n">
         <f aca="false">D28*E28</f>
-        <v>25280</v>
+        <v>25320</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1724,11 +1724,11 @@
         <v>4</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>6320</v>
+        <v>6330</v>
       </c>
       <c r="F29" s="5" t="n">
         <f aca="false">D29*E29</f>
-        <v>25280</v>
+        <v>25320</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1745,11 +1745,11 @@
         <v>4</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>6320</v>
+        <v>6330</v>
       </c>
       <c r="F30" s="5" t="n">
         <f aca="false">D30*E30</f>
-        <v>25280</v>
+        <v>25320</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1850,11 +1850,11 @@
         <v>3</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>7470</v>
+        <v>7480</v>
       </c>
       <c r="F35" s="5" t="n">
         <f aca="false">D35*E35</f>
-        <v>22410</v>
+        <v>22440</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1871,11 +1871,11 @@
         <v>3</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>12070</v>
+        <v>12080</v>
       </c>
       <c r="F36" s="5" t="n">
         <f aca="false">D36*E36</f>
-        <v>36210</v>
+        <v>36240</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1934,11 +1934,11 @@
         <v>3</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>4020</v>
+        <v>4030</v>
       </c>
       <c r="F39" s="5" t="n">
         <f aca="false">D39*E39</f>
-        <v>12060</v>
+        <v>12090</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2858,11 +2858,11 @@
         <v>1</v>
       </c>
       <c r="E83" s="5" t="n">
-        <v>7470</v>
+        <v>7480</v>
       </c>
       <c r="F83" s="5" t="n">
         <f aca="false">D83*E83</f>
-        <v>7470</v>
+        <v>7480</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2900,11 +2900,11 @@
         <v>1</v>
       </c>
       <c r="E85" s="5" t="n">
-        <v>14370</v>
+        <v>14380</v>
       </c>
       <c r="F85" s="5" t="n">
         <f aca="false">D85*E85</f>
-        <v>14370</v>
+        <v>14380</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2984,11 +2984,11 @@
         <v>2</v>
       </c>
       <c r="E89" s="5" t="n">
-        <v>7470</v>
+        <v>7480</v>
       </c>
       <c r="F89" s="5" t="n">
         <f aca="false">D89*E89</f>
-        <v>14940</v>
+        <v>14960</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3026,11 +3026,11 @@
         <v>2</v>
       </c>
       <c r="E91" s="5" t="n">
-        <v>4020</v>
+        <v>4030</v>
       </c>
       <c r="F91" s="5" t="n">
         <f aca="false">D91*E91</f>
-        <v>8040</v>
+        <v>8060</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3446,11 +3446,11 @@
         <v>3</v>
       </c>
       <c r="E111" s="5" t="n">
-        <v>6320</v>
+        <v>6330</v>
       </c>
       <c r="F111" s="5" t="n">
         <f aca="false">D111*E111</f>
-        <v>18960</v>
+        <v>18990</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4433,11 +4433,11 @@
         <v>150</v>
       </c>
       <c r="E158" s="5" t="n">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="F158" s="5" t="n">
         <f aca="false">D158*E158</f>
-        <v>17550</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4538,11 +4538,11 @@
         <v>20</v>
       </c>
       <c r="E163" s="5" t="n">
-        <v>3330</v>
+        <v>3340</v>
       </c>
       <c r="F163" s="5" t="n">
         <f aca="false">D163*E163</f>
-        <v>66600</v>
+        <v>66800</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4727,11 +4727,11 @@
         <v>3</v>
       </c>
       <c r="E172" s="5" t="n">
-        <v>3330</v>
+        <v>3340</v>
       </c>
       <c r="F172" s="5" t="n">
         <f aca="false">D172*E172</f>
-        <v>9990</v>
+        <v>10020</v>
       </c>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4748,11 +4748,11 @@
         <v>3</v>
       </c>
       <c r="E173" s="5" t="n">
-        <v>4020</v>
+        <v>4030</v>
       </c>
       <c r="F173" s="5" t="n">
         <f aca="false">D173*E173</f>
-        <v>12060</v>
+        <v>12090</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4832,11 +4832,11 @@
         <v>1</v>
       </c>
       <c r="E177" s="5" t="n">
-        <v>12070</v>
+        <v>12080</v>
       </c>
       <c r="F177" s="5" t="n">
         <f aca="false">D177*E177</f>
-        <v>12070</v>
+        <v>12080</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4916,11 +4916,11 @@
         <v>2</v>
       </c>
       <c r="E181" s="5" t="n">
-        <v>6320</v>
+        <v>6330</v>
       </c>
       <c r="F181" s="5" t="n">
         <f aca="false">D181*E181</f>
-        <v>12640</v>
+        <v>12660</v>
       </c>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4958,11 +4958,11 @@
         <v>2</v>
       </c>
       <c r="E183" s="5" t="n">
-        <v>6320</v>
+        <v>6330</v>
       </c>
       <c r="F183" s="5" t="n">
         <f aca="false">D183*E183</f>
-        <v>12640</v>
+        <v>12660</v>
       </c>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5147,11 +5147,11 @@
         <v>6</v>
       </c>
       <c r="E192" s="5" t="n">
-        <v>1490</v>
+        <v>1500</v>
       </c>
       <c r="F192" s="5" t="n">
         <f aca="false">D192*E192</f>
-        <v>8940</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5168,11 +5168,11 @@
         <v>6</v>
       </c>
       <c r="E193" s="5" t="n">
-        <v>1950</v>
+        <v>1960</v>
       </c>
       <c r="F193" s="5" t="n">
         <f aca="false">D193*E193</f>
-        <v>11700</v>
+        <v>11760</v>
       </c>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5315,11 +5315,11 @@
         <v>2</v>
       </c>
       <c r="E200" s="5" t="n">
-        <v>800</v>
+        <v>810</v>
       </c>
       <c r="F200" s="5" t="n">
         <f aca="false">D200*E200</f>
-        <v>1600</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5399,11 +5399,11 @@
         <v>2</v>
       </c>
       <c r="E204" s="5" t="n">
-        <v>1490</v>
+        <v>1500</v>
       </c>
       <c r="F204" s="5" t="n">
         <f aca="false">D204*E204</f>
-        <v>2980</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5441,11 +5441,11 @@
         <v>1</v>
       </c>
       <c r="E206" s="5" t="n">
-        <v>1720</v>
+        <v>1730</v>
       </c>
       <c r="F206" s="5" t="n">
         <f aca="false">D206*E206</f>
-        <v>1720</v>
+        <v>1730</v>
       </c>
     </row>
     <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5874,7 +5874,7 @@
       </c>
       <c r="F227" s="7" t="n">
         <f aca="false">SUM(F5:F226)</f>
-        <v>13973706</v>
+        <v>13975036</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use Pakistani online listings per item (Licota -> Yato -> other listed brand), add dealer RFQ sheets
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="257">
   <si>
     <t xml:space="preserve">Zidane Corporation - REVISED QUOTATION</t>
   </si>
@@ -76,303 +76,321 @@
     <t xml:space="preserve">SAFETY HELMET (WHITE)</t>
   </si>
   <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAFETY GOOGLES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue Eagle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7 DRAWER TOOL TROLLEY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOUBLE OPEN RING OFFSET WRENCH SET (12PCS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Harden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOUBLE OPEN END WRENCH 6 TO 32 (12 PCS SET)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOUBLE OPEN END WRENCH 36X41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Licota</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOUBLE OPEN END WRENCH 41X46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMBINATION WRENCH 8 TO 32 (14 PCS SET)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tolsen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOCKET SET (113PCS) 1/4" &amp; 1/2"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIN PUNCH SET (06PCS SET)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOLLOW PUNCH (3MM-25MM) (15PCS SET)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LONG TYPE HEX KEY WRENCH SET 09 PCS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SHORT TYPE HEX KEY WRENCH SET (09PCS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LONG TYPE HEX WRENCH SET 09 PCS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALLEN HEX KEY 12MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALLEN (HEX) KEY 14MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALLEN (HEX) KEY 16MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER INTERNAL STRAIGHT 175MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER INTERNAL BENT 175MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL STRAIGHT 175MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL BENT 175MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHISEL SET (05 PCS SET)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIPE WRENCH SIZE 10"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIPE WRENCH SIZE 12"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIPE WRENCH SIZE 18"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIPE WRENCH SIZE 24"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIPE WRENCH SIZE 36"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLEDGE HAMMER 3 LBS WITH FIBREGLASS HANDLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOFT FACE DEAD BLOW HAMMER 50MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VICE GRIP PLIER 08"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORDLESS IMPACT WRENCH 185NM (Bosch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bosch Professional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORDLESS IMPACT WRENCH 350N (Bosch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORDLESS IMPACT WRENCH 1000N (Bosch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLAT FILE 12"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROUNDE FILE 12"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIVERSAL PULLER 2-ARMED WITH HOOK BRAK 250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MECHANICAL PULLER 3 ARMED 200X200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MECHANICAL PULLER 3 ARMED 250X250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DRILL MACHINE CORDLESS ROTARY HAMMER Bosch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUAL GREASE GUN 5KG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AIR GREASE GUN 500CC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HAND GREASE GUN WITH HOSE 500CC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GREASE PIPE 1/4"X12"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOUBLE HANDLE GREASE NOZZLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STEEL MEASURMENT TAPE 100M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STEEL MEASURMENT TAPE 50M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADJUSTABLE WRENCH 15"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ROUGH FILE SMOOTH 10"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POLISH FILE SMOOTH 10"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REVOLVING CENTRE MT4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vertex (Taiwan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REVOLVING CENTRE MT3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCUMFERENCE TAPE (60-950) (D20-300)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insize</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCUMFERENCE TAPE (940-2200) (D300-700)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEASURING TAPE 5M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS COBALT DRILL SET 1-13MM 25 PCS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BITS 1/16-1/2" 29 PCS SET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 14MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dormer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 15MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 15.5MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 16MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 16.5MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 17MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 17.5MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 19MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 21MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 25MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 30MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 32MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 35MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEAD CENTRE DIAMOND TIP M2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEAD CENTRE DIAMOND TIP M3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIGITAL VERINER CALIPER 300MM (Insize brand)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUAL VERNIER CALLIPER 12" (Insize brand)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MANUAL VERNIER CALLIPER 8" (Insize (Bosch))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERNIER DEPTH GUAGE 250MM GRADUATION 0.02M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORDLESS DRILL DRIVER 150NM Bosch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAP SET 1/2" BSPF LEFT HAND (Dormer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAP SET 1/2" BSPF RIGHT HAND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAP SET 3/8" BSPF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAP SET 1/4" BSPF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TAP SET 1/8" BSPF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WIRE BRUSH HEAVY DUTY 4/5 NROW</t>
+  </si>
+  <si>
     <t xml:space="preserve">Industrial</t>
   </si>
   <si>
-    <t xml:space="preserve">SAFETY GOOGLES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7 DRAWER TOOL TROLLEY</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Licota</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOUBLE OPEN RING OFFSET WRENCH SET (12PCS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOUBLE OPEN END WRENCH 6 TO 32 (12 PCS SET)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOUBLE OPEN END WRENCH 36X41</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOUBLE OPEN END WRENCH 41X46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COMBINATION WRENCH 8 TO 32 (14 PCS SET)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOCKET SET (113PCS) 1/4" &amp; 1/2"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIN PUNCH SET (06PCS SET)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HOLLOW PUNCH (3MM-25MM) (15PCS SET)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LONG TYPE HEX KEY WRENCH SET 09 PCS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SHORT TYPE HEX KEY WRENCH SET (09PCS)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LONG TYPE HEX WRENCH SET 09 PCS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALLEN HEX KEY 12MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALLEN (HEX) KEY 14MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALLEN (HEX) KEY 16MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER INTERNAL STRAIGHT 175MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER INTERNAL BENT 175MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL STRAIGHT 175MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL BENT 175MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHISEL SET (05 PCS SET)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIPE WRENCH SIZE 10"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIPE WRENCH SIZE 12"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIPE WRENCH SIZE 18"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIPE WRENCH SIZE 24"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIPE WRENCH SIZE 36"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLEDGE HAMMER 3 LBS WITH FIBREGLASS HANDLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOFT FACE DEAD BLOW HAMMER 50MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VICE GRIP PLIER 08"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORDLESS IMPACT WRENCH 185NM (Bosch)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bosch Professional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORDLESS IMPACT WRENCH 350N (Bosch)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORDLESS IMPACT WRENCH 1000N (Bosch)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLAT FILE 12"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROUNDE FILE 12"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIVERSAL PULLER 2-ARMED WITH HOOK BRAKE 21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIVERSAL PULLER 2-ARMED WITH HOOK BRAK 250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIVERSAL PULLER 2-ARMED 160 X 300 MM 5T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIVERSAL PULLER 2-ARMED 250 X 300 MM 7.5T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INTERNAL EXTRACTOR WITH REINFORCED COLLAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MECHANICAL PULLER 3 ARMED 200X200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MECHANICAL PULLER 3 ARMED 250X250</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DRILL MACHINE CORDLESS ROTARY HAMMER Bosch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MANUAL GREASE GUN 5KG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AIR GREASE GUN 500CC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HAND GREASE GUN WITH HOSE 500CC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GREASE PIPE 1/4"X12"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DOUBLE HANDLE GREASE NOZZLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STEEL MEASURMENT TAPE 100M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">STEEL MEASURMENT TAPE 50M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ADJUSTABLE WRENCH 15"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ROUGH FILE SMOOTH 10"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">POLISH FILE SMOOTH 10"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REVOLVING CENTRE MT4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vertex (Taiwan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REVOLVING CENTRE MT3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCUMFERENCE TAPE (60-950) (D20-300)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Insize</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCUMFERENCE TAPE (940-2200) (D300-700)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEASURING TAPE 5M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS COBALT DRILL SET 1-13MM 25 PCS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BITS 1/16-1/2" 29 PCS SET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 14MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dormer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 15MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 15.5MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 16MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 16.5MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 17MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 17.5MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 19MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 21MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 25MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 30MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 32MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 35MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEAD CENTRE DIAMOND TIP M2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEAD CENTRE DIAMOND TIP M3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIGITAL VERINER CALIPER 300MM (Insize brand)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MANUAL VERNIER CALLIPER 12" (Insize brand)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MANUAL VERNIER CALLIPER 8" (Insize (Bosch))</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VERNIER DEPTH GUAGE 250MM GRADUATION 0.02M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORDLESS DRILL DRIVER 150NM Bosch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TAP SET 1/2" BSPF LEFT HAND (Dormer)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TAP SET 1/2" BSPF RIGHT HAND</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TAP SET 3/8" BSPF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TAP SET 1/4" BSPF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TAP SET 1/8" BSPF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">WIRE BRUSH HEAVY DUTY 4/5 NROW</t>
-  </si>
-  <si>
     <t xml:space="preserve">WELDING HELMET (FLIP FRONT)</t>
   </si>
   <si>
     <t xml:space="preserve">WELDING LEATHER GLOVES 16"</t>
   </si>
   <si>
+    <t xml:space="preserve">Leather Forge</t>
+  </si>
+  <si>
     <t xml:space="preserve">C-CLAMP 6"</t>
   </si>
   <si>
@@ -403,6 +421,9 @@
     <t xml:space="preserve">OXYGEN REGULATOR 0-10 BAR</t>
   </si>
   <si>
+    <t xml:space="preserve">Tanaka</t>
+  </si>
+  <si>
     <t xml:space="preserve">FUEL GAS REGULATOR 0-2.5 BAR</t>
   </si>
   <si>
@@ -451,6 +472,9 @@
     <t xml:space="preserve">ARGON REGULATOR FLOW METER</t>
   </si>
   <si>
+    <t xml:space="preserve">WM</t>
+  </si>
+  <si>
     <t xml:space="preserve">ARGON GAS HOSE 06MM</t>
   </si>
   <si>
@@ -496,6 +520,9 @@
     <t xml:space="preserve">HYDRAULIC HAND TROLLY 3T</t>
   </si>
   <si>
+    <t xml:space="preserve">VMAX</t>
+  </si>
+  <si>
     <t xml:space="preserve">HYDRAULIC HAND TROLLY 5T</t>
   </si>
   <si>
@@ -526,12 +553,18 @@
     <t xml:space="preserve">SPRAY WHITE</t>
   </si>
   <si>
+    <t xml:space="preserve">7CF</t>
+  </si>
+  <si>
     <t xml:space="preserve">SPRAY BLUE</t>
   </si>
   <si>
     <t xml:space="preserve">SPRAY GREEN</t>
   </si>
   <si>
+    <t xml:space="preserve">Mubah</t>
+  </si>
+  <si>
     <t xml:space="preserve">TOILET CLEANING BRUSH</t>
   </si>
   <si>
@@ -550,12 +583,18 @@
     <t xml:space="preserve">WELDING RODS 2.5MM E6013, NO 10 Zodian</t>
   </si>
   <si>
+    <t xml:space="preserve">Zodian</t>
+  </si>
+  <si>
     <t xml:space="preserve">WELDING RODS 3.25MM E6013 NO 12</t>
   </si>
   <si>
     <t xml:space="preserve">WELDING RODS 2.5MM E7018 NO-10</t>
   </si>
   <si>
+    <t xml:space="preserve">Fortrex</t>
+  </si>
+  <si>
     <t xml:space="preserve">SS WELDING RODS 309L-16 2.6MM NO.12</t>
   </si>
   <si>
@@ -716,6 +755,9 @@
   </si>
   <si>
     <t xml:space="preserve">HYDRAULIC JACK 3 TON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ronix</t>
   </si>
   <si>
     <t xml:space="preserve">HYDRAULIC JACK 5 TON</t>
@@ -1325,11 +1367,11 @@
         <v>6</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>1150</v>
+        <v>1105</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">D10*E10</f>
-        <v>6900</v>
+        <v>6630</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1340,7 +1382,7 @@
         <v>19</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>24</v>
@@ -1358,20 +1400,20 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>241500</v>
+        <v>117450</v>
       </c>
       <c r="F12" s="5" t="n">
         <f aca="false">D12*E12</f>
-        <v>724500</v>
+        <v>352350</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1382,17 +1424,17 @@
         <v>22</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>29900</v>
+        <v>18200</v>
       </c>
       <c r="F13" s="5" t="n">
         <f aca="false">D13*E13</f>
-        <v>119600</v>
+        <v>72800</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1400,20 +1442,20 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>24150</v>
+        <v>15600</v>
       </c>
       <c r="F14" s="5" t="n">
         <f aca="false">D14*E14</f>
-        <v>96600</v>
+        <v>62400</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1421,10 +1463,10 @@
         <v>11</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>3</v>
@@ -1442,10 +1484,10 @@
         <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>3</v>
@@ -1463,20 +1505,20 @@
         <v>13</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>34500</v>
+        <v>15900</v>
       </c>
       <c r="F17" s="5" t="n">
         <f aca="false">D17*E17</f>
-        <v>138000</v>
+        <v>63600</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1484,20 +1526,20 @@
         <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>77280</v>
+        <v>77200</v>
       </c>
       <c r="F18" s="5" t="n">
         <f aca="false">D18*E18</f>
-        <v>309120</v>
+        <v>308800</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1505,20 +1547,20 @@
         <v>15</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>7130</v>
+        <v>6280</v>
       </c>
       <c r="F19" s="5" t="n">
         <f aca="false">D19*E19</f>
-        <v>28520</v>
+        <v>25120</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1526,20 +1568,20 @@
         <v>16</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>10350</v>
+        <v>8450</v>
       </c>
       <c r="F20" s="5" t="n">
         <f aca="false">D20*E20</f>
-        <v>41400</v>
+        <v>33800</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1547,10 +1589,10 @@
         <v>17</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>4</v>
@@ -1568,20 +1610,20 @@
         <v>18</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D22" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>3450</v>
+        <v>1846</v>
       </c>
       <c r="F22" s="5" t="n">
         <f aca="false">D22*E22</f>
-        <v>13800</v>
+        <v>7384</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1589,10 +1631,10 @@
         <v>19</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>4</v>
@@ -1610,10 +1652,10 @@
         <v>20</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D24" s="4" t="n">
         <v>3</v>
@@ -1631,10 +1673,10 @@
         <v>21</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D25" s="4" t="n">
         <v>3</v>
@@ -1652,10 +1694,10 @@
         <v>22</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D26" s="4" t="n">
         <v>3</v>
@@ -1673,20 +1715,20 @@
         <v>23</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D27" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E27" s="5" t="n">
-        <v>6330</v>
+        <v>4940</v>
       </c>
       <c r="F27" s="5" t="n">
         <f aca="false">D27*E27</f>
-        <v>25320</v>
+        <v>19760</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1694,20 +1736,20 @@
         <v>24</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D28" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E28" s="5" t="n">
-        <v>6330</v>
+        <v>4940</v>
       </c>
       <c r="F28" s="5" t="n">
         <f aca="false">D28*E28</f>
-        <v>25320</v>
+        <v>19760</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1715,20 +1757,20 @@
         <v>25</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D29" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>6330</v>
+        <v>4940</v>
       </c>
       <c r="F29" s="5" t="n">
         <f aca="false">D29*E29</f>
-        <v>25320</v>
+        <v>19760</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1736,20 +1778,20 @@
         <v>26</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D30" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>6330</v>
+        <v>4940</v>
       </c>
       <c r="F30" s="5" t="n">
         <f aca="false">D30*E30</f>
-        <v>25320</v>
+        <v>19760</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1757,10 +1799,10 @@
         <v>27</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D31" s="4" t="n">
         <v>4</v>
@@ -1778,10 +1820,10 @@
         <v>28</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D32" s="4" t="n">
         <v>3</v>
@@ -1799,10 +1841,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D33" s="4" t="n">
         <v>4</v>
@@ -1820,20 +1862,20 @@
         <v>31</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D34" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>5980</v>
+        <v>2210</v>
       </c>
       <c r="F34" s="5" t="n">
         <f aca="false">D34*E34</f>
-        <v>17940</v>
+        <v>6630</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1841,20 +1883,20 @@
         <v>32</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D35" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>7480</v>
+        <v>3280</v>
       </c>
       <c r="F35" s="5" t="n">
         <f aca="false">D35*E35</f>
-        <v>22440</v>
+        <v>9840</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1862,20 +1904,20 @@
         <v>33</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D36" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>12080</v>
+        <v>11060</v>
       </c>
       <c r="F36" s="5" t="n">
         <f aca="false">D36*E36</f>
-        <v>36240</v>
+        <v>33180</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1883,20 +1925,20 @@
         <v>34</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D37" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>18400</v>
+        <v>7540</v>
       </c>
       <c r="F37" s="5" t="n">
         <f aca="false">D37*E37</f>
-        <v>36800</v>
+        <v>15080</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1904,20 +1946,20 @@
         <v>35</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D38" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>32200</v>
+        <v>12870</v>
       </c>
       <c r="F38" s="5" t="n">
         <f aca="false">D38*E38</f>
-        <v>64400</v>
+        <v>25740</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1925,20 +1967,20 @@
         <v>36</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D39" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>4030</v>
+        <v>2300</v>
       </c>
       <c r="F39" s="5" t="n">
         <f aca="false">D39*E39</f>
-        <v>12090</v>
+        <v>6900</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1946,20 +1988,20 @@
         <v>37</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D40" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>6900</v>
+        <v>4550</v>
       </c>
       <c r="F40" s="5" t="n">
         <f aca="false">D40*E40</f>
-        <v>20700</v>
+        <v>13650</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1967,20 +2009,20 @@
         <v>38</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D41" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>8050</v>
+        <v>3310</v>
       </c>
       <c r="F41" s="5" t="n">
         <f aca="false">D41*E41</f>
-        <v>24150</v>
+        <v>9930</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1988,10 +2030,10 @@
         <v>39</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D42" s="4" t="n">
         <v>3</v>
@@ -2009,10 +2051,10 @@
         <v>40</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D43" s="4" t="n">
         <v>3</v>
@@ -2030,10 +2072,10 @@
         <v>41</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D44" s="4" t="n">
         <v>3</v>
@@ -2051,10 +2093,10 @@
         <v>42</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D45" s="4" t="n">
         <v>2</v>
@@ -2072,10 +2114,10 @@
         <v>43</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D46" s="4" t="n">
         <v>4</v>
@@ -2093,7 +2135,7 @@
         <v>44</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>15</v>
@@ -2102,11 +2144,11 @@
         <v>4</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>2300</v>
+        <v>2010</v>
       </c>
       <c r="F47" s="5" t="n">
         <f aca="false">D47*E47</f>
-        <v>9200</v>
+        <v>8040</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2114,7 +2156,7 @@
         <v>45</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>15</v>
@@ -2135,10 +2177,10 @@
         <v>47</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D49" s="4" t="n">
         <v>3</v>
@@ -2156,10 +2198,10 @@
         <v>48</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D50" s="4" t="n">
         <v>2</v>
@@ -2177,10 +2219,10 @@
         <v>49</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D51" s="4" t="n">
         <v>1</v>
@@ -2198,10 +2240,10 @@
         <v>50</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D52" s="4" t="n">
         <v>1</v>
@@ -2219,10 +2261,10 @@
         <v>51</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D53" s="4" t="n">
         <v>1</v>
@@ -2240,20 +2282,20 @@
         <v>52</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D54" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>28750</v>
+        <v>11480</v>
       </c>
       <c r="F54" s="5" t="n">
         <f aca="false">D54*E54</f>
-        <v>57500</v>
+        <v>22960</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2261,20 +2303,20 @@
         <v>53</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="D55" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>36800</v>
+        <v>23400</v>
       </c>
       <c r="F55" s="5" t="n">
         <f aca="false">D55*E55</f>
-        <v>36800</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2282,10 +2324,10 @@
         <v>54</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D56" s="4" t="n">
         <v>2</v>
@@ -2303,7 +2345,7 @@
         <v>55</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>15</v>
@@ -2324,10 +2366,10 @@
         <v>56</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D58" s="4" t="n">
         <v>1</v>
@@ -2345,20 +2387,20 @@
         <v>57</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D59" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>10350</v>
+        <v>8920</v>
       </c>
       <c r="F59" s="5" t="n">
         <f aca="false">D59*E59</f>
-        <v>41400</v>
+        <v>35680</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2366,10 +2408,10 @@
         <v>58</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D60" s="4" t="n">
         <v>12</v>
@@ -2387,10 +2429,10 @@
         <v>59</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D61" s="4" t="n">
         <v>12</v>
@@ -2408,7 +2450,7 @@
         <v>60</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C62" s="4" t="s">
         <v>15</v>
@@ -2429,20 +2471,20 @@
         <v>61</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
       <c r="D63" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>8630</v>
+        <v>6810</v>
       </c>
       <c r="F63" s="5" t="n">
         <f aca="false">D63*E63</f>
-        <v>17260</v>
+        <v>13620</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2450,10 +2492,10 @@
         <v>62</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="D64" s="4" t="n">
         <v>3</v>
@@ -2471,20 +2513,20 @@
         <v>63</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D65" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>12650</v>
+        <v>5551</v>
       </c>
       <c r="F65" s="5" t="n">
         <f aca="false">D65*E65</f>
-        <v>12650</v>
+        <v>5551</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2492,7 +2534,7 @@
         <v>64</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C66" s="4" t="s">
         <v>15</v>
@@ -2501,11 +2543,11 @@
         <v>3</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>1840</v>
+        <v>1560</v>
       </c>
       <c r="F66" s="5" t="n">
         <f aca="false">D66*E66</f>
-        <v>5520</v>
+        <v>4680</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2513,7 +2555,7 @@
         <v>65</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="C67" s="4" t="s">
         <v>15</v>
@@ -2522,11 +2564,11 @@
         <v>3</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>1840</v>
+        <v>1560</v>
       </c>
       <c r="F67" s="5" t="n">
         <f aca="false">D67*E67</f>
-        <v>5520</v>
+        <v>4680</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2534,10 +2576,10 @@
         <v>66</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D68" s="4" t="n">
         <v>2</v>
@@ -2555,10 +2597,10 @@
         <v>67</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D69" s="4" t="n">
         <v>2</v>
@@ -2576,10 +2618,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D70" s="4" t="n">
         <v>2</v>
@@ -2597,10 +2639,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D71" s="4" t="n">
         <v>1</v>
@@ -2618,20 +2660,20 @@
         <v>71</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D72" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E72" s="5" t="n">
-        <v>1380</v>
+        <v>1150</v>
       </c>
       <c r="F72" s="5" t="n">
         <f aca="false">D72*E72</f>
-        <v>1380</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2639,20 +2681,20 @@
         <v>73</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
       <c r="D73" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E73" s="5" t="n">
-        <v>45500</v>
+        <v>29950</v>
       </c>
       <c r="F73" s="5" t="n">
         <f aca="false">D73*E73</f>
-        <v>45500</v>
+        <v>29950</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2660,7 +2702,7 @@
         <v>74</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>15</v>
@@ -2681,10 +2723,10 @@
         <v>75</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D75" s="4" t="n">
         <v>2</v>
@@ -2702,10 +2744,10 @@
         <v>76</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D76" s="4" t="n">
         <v>2</v>
@@ -2723,10 +2765,10 @@
         <v>77</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D77" s="4" t="n">
         <v>2</v>
@@ -2744,10 +2786,10 @@
         <v>78</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D78" s="4" t="n">
         <v>2</v>
@@ -2765,10 +2807,10 @@
         <v>79</v>
       </c>
       <c r="B79" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C79" s="4" t="s">
         <v>92</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>88</v>
       </c>
       <c r="D79" s="4" t="n">
         <v>2</v>
@@ -2786,10 +2828,10 @@
         <v>80</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D80" s="4" t="n">
         <v>2</v>
@@ -2807,10 +2849,10 @@
         <v>81</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D81" s="4" t="n">
         <v>2</v>
@@ -2828,10 +2870,10 @@
         <v>82</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D82" s="4" t="n">
         <v>2</v>
@@ -2849,10 +2891,10 @@
         <v>83</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D83" s="4" t="n">
         <v>1</v>
@@ -2870,10 +2912,10 @@
         <v>84</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D84" s="4" t="n">
         <v>1</v>
@@ -2891,10 +2933,10 @@
         <v>85</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D85" s="4" t="n">
         <v>1</v>
@@ -2912,10 +2954,10 @@
         <v>86</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D86" s="4" t="n">
         <v>1</v>
@@ -2933,10 +2975,10 @@
         <v>87</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D87" s="4" t="n">
         <v>1</v>
@@ -2954,10 +2996,10 @@
         <v>88</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D88" s="4" t="n">
         <v>2</v>
@@ -2975,10 +3017,10 @@
         <v>89</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D89" s="4" t="n">
         <v>2</v>
@@ -2996,10 +3038,10 @@
         <v>90</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D90" s="4" t="n">
         <v>2</v>
@@ -3017,10 +3059,10 @@
         <v>91</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D91" s="4" t="n">
         <v>2</v>
@@ -3038,10 +3080,10 @@
         <v>92</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D92" s="4" t="n">
         <v>2</v>
@@ -3059,10 +3101,10 @@
         <v>93</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D93" s="4" t="n">
         <v>2</v>
@@ -3080,20 +3122,20 @@
         <v>94</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D94" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E94" s="5" t="n">
-        <v>21740</v>
+        <v>18170</v>
       </c>
       <c r="F94" s="5" t="n">
         <f aca="false">D94*E94</f>
-        <v>65220</v>
+        <v>54510</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3101,20 +3143,20 @@
         <v>95</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D95" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E95" s="5" t="n">
-        <v>10120</v>
+        <v>9120</v>
       </c>
       <c r="F95" s="5" t="n">
         <f aca="false">D95*E95</f>
-        <v>30360</v>
+        <v>27360</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3122,10 +3164,10 @@
         <v>96</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D96" s="4" t="n">
         <v>2</v>
@@ -3143,10 +3185,10 @@
         <v>97</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D97" s="4" t="n">
         <v>2</v>
@@ -3164,10 +3206,10 @@
         <v>98</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D98" s="4" t="n">
         <v>1</v>
@@ -3185,10 +3227,10 @@
         <v>99</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D99" s="4" t="n">
         <v>1</v>
@@ -3206,10 +3248,10 @@
         <v>100</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D100" s="4" t="n">
         <v>1</v>
@@ -3227,10 +3269,10 @@
         <v>101</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D101" s="4" t="n">
         <v>3</v>
@@ -3248,10 +3290,10 @@
         <v>102</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D102" s="4" t="n">
         <v>3</v>
@@ -3269,10 +3311,10 @@
         <v>103</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D103" s="4" t="n">
         <v>12</v>
@@ -3290,10 +3332,10 @@
         <v>104</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D104" s="4" t="n">
         <v>4</v>
@@ -3311,10 +3353,10 @@
         <v>105</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>18</v>
+        <v>122</v>
       </c>
       <c r="D105" s="4" t="n">
         <v>12</v>
@@ -3332,10 +3374,10 @@
         <v>106</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D106" s="4" t="n">
         <v>6</v>
@@ -3353,7 +3395,7 @@
         <v>107</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C107" s="4" t="s">
         <v>15</v>
@@ -3374,20 +3416,20 @@
         <v>108</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D108" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E108" s="5" t="n">
-        <v>5750</v>
+        <v>4550</v>
       </c>
       <c r="F108" s="5" t="n">
         <f aca="false">D108*E108</f>
-        <v>17250</v>
+        <v>13650</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3395,7 +3437,7 @@
         <v>109</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C109" s="4" t="s">
         <v>15</v>
@@ -3416,10 +3458,10 @@
         <v>110</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D110" s="4" t="n">
         <v>3</v>
@@ -3437,20 +3479,20 @@
         <v>111</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>82</v>
+        <v>23</v>
       </c>
       <c r="D111" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E111" s="5" t="n">
-        <v>6330</v>
+        <v>3590</v>
       </c>
       <c r="F111" s="5" t="n">
         <f aca="false">D111*E111</f>
-        <v>18990</v>
+        <v>10770</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3458,10 +3500,10 @@
         <v>112</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D112" s="4" t="n">
         <v>2</v>
@@ -3479,10 +3521,10 @@
         <v>113</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D113" s="4" t="n">
         <v>3</v>
@@ -3500,10 +3542,10 @@
         <v>114</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D114" s="4" t="n">
         <v>3</v>
@@ -3521,20 +3563,20 @@
         <v>115</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>18</v>
+        <v>133</v>
       </c>
       <c r="D115" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E115" s="5" t="n">
-        <v>11050</v>
+        <v>6750</v>
       </c>
       <c r="F115" s="5" t="n">
         <f aca="false">D115*E115</f>
-        <v>22100</v>
+        <v>13500</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3542,10 +3584,10 @@
         <v>116</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D116" s="4" t="n">
         <v>2</v>
@@ -3563,10 +3605,10 @@
         <v>117</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D117" s="4" t="n">
         <v>15</v>
@@ -3584,10 +3626,10 @@
         <v>118</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D118" s="4" t="n">
         <v>15</v>
@@ -3605,10 +3647,10 @@
         <v>119</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D119" s="4" t="n">
         <v>2</v>
@@ -3626,10 +3668,10 @@
         <v>120</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D120" s="4" t="n">
         <v>6</v>
@@ -3647,7 +3689,7 @@
         <v>121</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C121" s="4" t="s">
         <v>18</v>
@@ -3656,11 +3698,11 @@
         <v>6</v>
       </c>
       <c r="E121" s="5" t="n">
-        <v>637</v>
+        <v>690</v>
       </c>
       <c r="F121" s="5" t="n">
         <f aca="false">D121*E121</f>
-        <v>3822</v>
+        <v>4140</v>
       </c>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3668,10 +3710,10 @@
         <v>122</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D122" s="4" t="n">
         <v>1</v>
@@ -3689,10 +3731,10 @@
         <v>123</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D123" s="4" t="n">
         <v>2</v>
@@ -3710,10 +3752,10 @@
         <v>124</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D124" s="4" t="n">
         <v>2</v>
@@ -3731,10 +3773,10 @@
         <v>125</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D125" s="4" t="n">
         <v>12</v>
@@ -3752,10 +3794,10 @@
         <v>126</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D126" s="4" t="n">
         <v>12</v>
@@ -3773,10 +3815,10 @@
         <v>127</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D127" s="4" t="n">
         <v>6</v>
@@ -3794,10 +3836,10 @@
         <v>128</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D128" s="4" t="n">
         <v>6</v>
@@ -3815,10 +3857,10 @@
         <v>129</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D129" s="4" t="n">
         <v>6</v>
@@ -3836,10 +3878,10 @@
         <v>130</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D130" s="4" t="n">
         <v>6</v>
@@ -3857,10 +3899,10 @@
         <v>131</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>18</v>
+        <v>150</v>
       </c>
       <c r="D131" s="4" t="n">
         <v>2</v>
@@ -3878,10 +3920,10 @@
         <v>132</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D132" s="4" t="n">
         <v>10</v>
@@ -3899,10 +3941,10 @@
         <v>133</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D133" s="4" t="n">
         <v>6</v>
@@ -3920,10 +3962,10 @@
         <v>134</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D134" s="4" t="n">
         <v>6</v>
@@ -3941,7 +3983,7 @@
         <v>135</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="C135" s="4" t="s">
         <v>18</v>
@@ -3950,11 +3992,11 @@
         <v>6</v>
       </c>
       <c r="E135" s="5" t="n">
-        <v>2880</v>
+        <v>1340</v>
       </c>
       <c r="F135" s="5" t="n">
         <f aca="false">D135*E135</f>
-        <v>17280</v>
+        <v>8040</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3962,7 +4004,7 @@
         <v>136</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="C136" s="4" t="s">
         <v>18</v>
@@ -3983,7 +4025,7 @@
         <v>138</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="C137" s="4" t="s">
         <v>18</v>
@@ -3992,11 +4034,11 @@
         <v>24</v>
       </c>
       <c r="E137" s="5" t="n">
-        <v>1170</v>
+        <v>800</v>
       </c>
       <c r="F137" s="5" t="n">
         <f aca="false">D137*E137</f>
-        <v>28080</v>
+        <v>19200</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4004,10 +4046,10 @@
         <v>139</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D138" s="4" t="n">
         <v>24</v>
@@ -4025,10 +4067,10 @@
         <v>140</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D139" s="4" t="n">
         <v>24</v>
@@ -4046,10 +4088,10 @@
         <v>142</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="D140" s="4" t="n">
         <v>3</v>
@@ -4067,10 +4109,10 @@
         <v>143</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="D141" s="4" t="n">
         <v>3</v>
@@ -4088,10 +4130,10 @@
         <v>144</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="D142" s="4" t="n">
         <v>3</v>
@@ -4109,10 +4151,10 @@
         <v>145</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="D143" s="4" t="n">
         <v>500</v>
@@ -4130,10 +4172,10 @@
         <v>146</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="C144" s="4" t="s">
-        <v>18</v>
+        <v>166</v>
       </c>
       <c r="D144" s="4" t="n">
         <v>1</v>
@@ -4151,10 +4193,10 @@
         <v>147</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>18</v>
+        <v>166</v>
       </c>
       <c r="D145" s="4" t="n">
         <v>1</v>
@@ -4172,20 +4214,20 @@
         <v>148</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="C146" s="4" t="s">
-        <v>156</v>
+        <v>29</v>
       </c>
       <c r="D146" s="4" t="n">
         <v>12</v>
       </c>
       <c r="E146" s="5" t="n">
-        <v>650</v>
+        <v>490</v>
       </c>
       <c r="F146" s="5" t="n">
         <f aca="false">D146*E146</f>
-        <v>7800</v>
+        <v>5880</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4193,10 +4235,10 @@
         <v>149</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="D147" s="4" t="n">
         <v>100</v>
@@ -4214,7 +4256,7 @@
         <v>150</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="C148" s="4" t="s">
         <v>18</v>
@@ -4235,7 +4277,7 @@
         <v>151</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="C149" s="4" t="s">
         <v>18</v>
@@ -4244,11 +4286,11 @@
         <v>100</v>
       </c>
       <c r="E149" s="5" t="n">
-        <v>650</v>
+        <v>680</v>
       </c>
       <c r="F149" s="5" t="n">
         <f aca="false">D149*E149</f>
-        <v>65000</v>
+        <v>68000</v>
       </c>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4256,7 +4298,7 @@
         <v>152</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="C150" s="4" t="s">
         <v>18</v>
@@ -4265,11 +4307,11 @@
         <v>24</v>
       </c>
       <c r="E150" s="5" t="n">
-        <v>546</v>
+        <v>630</v>
       </c>
       <c r="F150" s="5" t="n">
         <f aca="false">D150*E150</f>
-        <v>13104</v>
+        <v>15120</v>
       </c>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4277,7 +4319,7 @@
         <v>153</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="C151" s="4" t="s">
         <v>18</v>
@@ -4286,11 +4328,11 @@
         <v>24</v>
       </c>
       <c r="E151" s="5" t="n">
-        <v>1150</v>
+        <v>1105</v>
       </c>
       <c r="F151" s="5" t="n">
         <f aca="false">D151*E151</f>
-        <v>27600</v>
+        <v>26520</v>
       </c>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4298,10 +4340,10 @@
         <v>154</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D152" s="4" t="n">
         <v>12</v>
@@ -4319,10 +4361,10 @@
         <v>155</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>18</v>
+        <v>177</v>
       </c>
       <c r="D153" s="4" t="n">
         <v>50</v>
@@ -4340,10 +4382,10 @@
         <v>156</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>18</v>
+        <v>177</v>
       </c>
       <c r="D154" s="4" t="n">
         <v>30</v>
@@ -4361,20 +4403,20 @@
         <v>157</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>18</v>
+        <v>180</v>
       </c>
       <c r="D155" s="4" t="n">
         <v>30</v>
       </c>
       <c r="E155" s="5" t="n">
-        <v>748</v>
+        <v>540</v>
       </c>
       <c r="F155" s="5" t="n">
         <f aca="false">D155*E155</f>
-        <v>22440</v>
+        <v>16200</v>
       </c>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4382,10 +4424,10 @@
         <v>158</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>170</v>
+        <v>181</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="D156" s="4" t="n">
         <v>12</v>
@@ -4403,10 +4445,10 @@
         <v>159</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="D157" s="4" t="n">
         <v>100</v>
@@ -4424,10 +4466,10 @@
         <v>160</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="D158" s="4" t="n">
         <v>150</v>
@@ -4445,10 +4487,10 @@
         <v>161</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="D159" s="4" t="n">
         <v>150</v>
@@ -4466,10 +4508,10 @@
         <v>162</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="D160" s="4" t="n">
         <v>150</v>
@@ -4487,20 +4529,20 @@
         <v>164</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>18</v>
+        <v>187</v>
       </c>
       <c r="D161" s="4" t="n">
         <v>40</v>
       </c>
       <c r="E161" s="5" t="n">
-        <v>1270</v>
+        <v>1670</v>
       </c>
       <c r="F161" s="5" t="n">
         <f aca="false">D161*E161</f>
-        <v>50800</v>
+        <v>66800</v>
       </c>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4508,20 +4550,20 @@
         <v>165</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>18</v>
+        <v>187</v>
       </c>
       <c r="D162" s="4" t="n">
         <v>40</v>
       </c>
       <c r="E162" s="5" t="n">
-        <v>1270</v>
+        <v>2590</v>
       </c>
       <c r="F162" s="5" t="n">
         <f aca="false">D162*E162</f>
-        <v>50800</v>
+        <v>103600</v>
       </c>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4529,20 +4571,20 @@
         <v>166</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>18</v>
+        <v>190</v>
       </c>
       <c r="D163" s="4" t="n">
         <v>20</v>
       </c>
       <c r="E163" s="5" t="n">
-        <v>3340</v>
+        <v>3022</v>
       </c>
       <c r="F163" s="5" t="n">
         <f aca="false">D163*E163</f>
-        <v>66800</v>
+        <v>60440</v>
       </c>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4550,10 +4592,10 @@
         <v>167</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="C164" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D164" s="4" t="n">
         <v>40</v>
@@ -4571,10 +4613,10 @@
         <v>168</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="C165" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D165" s="4" t="n">
         <v>20</v>
@@ -4592,10 +4634,10 @@
         <v>177</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="C166" s="4" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="D166" s="4" t="n">
         <v>3</v>
@@ -4613,10 +4655,10 @@
         <v>179</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>181</v>
+        <v>194</v>
       </c>
       <c r="C167" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D167" s="4" t="n">
         <v>1</v>
@@ -4634,10 +4676,10 @@
         <v>180</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>182</v>
+        <v>195</v>
       </c>
       <c r="C168" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D168" s="4" t="n">
         <v>1</v>
@@ -4655,10 +4697,10 @@
         <v>181</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>183</v>
+        <v>196</v>
       </c>
       <c r="C169" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D169" s="4" t="n">
         <v>1</v>
@@ -4676,10 +4718,10 @@
         <v>182</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="C170" s="4" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D170" s="4" t="n">
         <v>1</v>
@@ -4697,7 +4739,7 @@
         <v>183</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="C171" s="4" t="s">
         <v>15</v>
@@ -4718,7 +4760,7 @@
         <v>184</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>186</v>
+        <v>199</v>
       </c>
       <c r="C172" s="4" t="s">
         <v>15</v>
@@ -4739,7 +4781,7 @@
         <v>185</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="C173" s="4" t="s">
         <v>15</v>
@@ -4760,7 +4802,7 @@
         <v>186</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="C174" s="4" t="s">
         <v>15</v>
@@ -4781,7 +4823,7 @@
         <v>187</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="C175" s="4" t="s">
         <v>15</v>
@@ -4802,7 +4844,7 @@
         <v>188</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="C176" s="4" t="s">
         <v>15</v>
@@ -4823,7 +4865,7 @@
         <v>189</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="C177" s="4" t="s">
         <v>15</v>
@@ -4844,7 +4886,7 @@
         <v>190</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="C178" s="4" t="s">
         <v>15</v>
@@ -4865,7 +4907,7 @@
         <v>191</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="C179" s="4" t="s">
         <v>15</v>
@@ -4886,7 +4928,7 @@
         <v>192</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>193</v>
+        <v>206</v>
       </c>
       <c r="C180" s="4" t="s">
         <v>11</v>
@@ -4907,7 +4949,7 @@
         <v>193</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>194</v>
+        <v>207</v>
       </c>
       <c r="C181" s="4" t="s">
         <v>11</v>
@@ -4928,7 +4970,7 @@
         <v>194</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>195</v>
+        <v>208</v>
       </c>
       <c r="C182" s="4" t="s">
         <v>11</v>
@@ -4949,7 +4991,7 @@
         <v>195</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="C183" s="4" t="s">
         <v>11</v>
@@ -4970,7 +5012,7 @@
         <v>196</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>197</v>
+        <v>210</v>
       </c>
       <c r="C184" s="4" t="s">
         <v>15</v>
@@ -4991,10 +5033,10 @@
         <v>197</v>
       </c>
       <c r="B185" s="4" t="s">
-        <v>198</v>
+        <v>211</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D185" s="4" t="n">
         <v>1</v>
@@ -5012,20 +5054,20 @@
         <v>198</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>199</v>
+        <v>212</v>
       </c>
       <c r="C186" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D186" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E186" s="5" t="n">
-        <v>8780</v>
+        <v>7430</v>
       </c>
       <c r="F186" s="5" t="n">
         <f aca="false">D186*E186</f>
-        <v>8780</v>
+        <v>7430</v>
       </c>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5033,20 +5075,20 @@
         <v>199</v>
       </c>
       <c r="B187" s="4" t="s">
-        <v>200</v>
+        <v>213</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D187" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E187" s="5" t="n">
-        <v>9720</v>
+        <v>8370</v>
       </c>
       <c r="F187" s="5" t="n">
         <f aca="false">D187*E187</f>
-        <v>9720</v>
+        <v>8370</v>
       </c>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5054,20 +5096,20 @@
         <v>200</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>201</v>
+        <v>214</v>
       </c>
       <c r="C188" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D188" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E188" s="5" t="n">
-        <v>10530</v>
+        <v>9280</v>
       </c>
       <c r="F188" s="5" t="n">
         <f aca="false">D188*E188</f>
-        <v>10530</v>
+        <v>9280</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5075,20 +5117,20 @@
         <v>201</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>202</v>
+        <v>215</v>
       </c>
       <c r="C189" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D189" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E189" s="5" t="n">
-        <v>13230</v>
+        <v>11810</v>
       </c>
       <c r="F189" s="5" t="n">
         <f aca="false">D189*E189</f>
-        <v>13230</v>
+        <v>11810</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5096,7 +5138,7 @@
         <v>202</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
       <c r="C190" s="4" t="s">
         <v>15</v>
@@ -5117,10 +5159,10 @@
         <v>204</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="C191" s="4" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D191" s="4" t="n">
         <v>6</v>
@@ -5138,10 +5180,10 @@
         <v>205</v>
       </c>
       <c r="B192" s="4" t="s">
-        <v>206</v>
+        <v>219</v>
       </c>
       <c r="C192" s="4" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D192" s="4" t="n">
         <v>6</v>
@@ -5159,10 +5201,10 @@
         <v>206</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>207</v>
+        <v>220</v>
       </c>
       <c r="C193" s="4" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D193" s="4" t="n">
         <v>6</v>
@@ -5180,10 +5222,10 @@
         <v>207</v>
       </c>
       <c r="B194" s="4" t="s">
-        <v>208</v>
+        <v>221</v>
       </c>
       <c r="C194" s="4" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D194" s="4" t="n">
         <v>4</v>
@@ -5201,10 +5243,10 @@
         <v>208</v>
       </c>
       <c r="B195" s="4" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="C195" s="4" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D195" s="4" t="n">
         <v>3</v>
@@ -5222,10 +5264,10 @@
         <v>209</v>
       </c>
       <c r="B196" s="4" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="C196" s="4" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D196" s="4" t="n">
         <v>3</v>
@@ -5243,10 +5285,10 @@
         <v>210</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="C197" s="4" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D197" s="4" t="n">
         <v>2</v>
@@ -5264,10 +5306,10 @@
         <v>211</v>
       </c>
       <c r="B198" s="4" t="s">
-        <v>212</v>
+        <v>225</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D198" s="4" t="n">
         <v>1</v>
@@ -5285,10 +5327,10 @@
         <v>212</v>
       </c>
       <c r="B199" s="4" t="s">
-        <v>213</v>
+        <v>226</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D199" s="4" t="n">
         <v>1</v>
@@ -5306,7 +5348,7 @@
         <v>213</v>
       </c>
       <c r="B200" s="4" t="s">
-        <v>214</v>
+        <v>227</v>
       </c>
       <c r="C200" s="4" t="s">
         <v>15</v>
@@ -5327,7 +5369,7 @@
         <v>214</v>
       </c>
       <c r="B201" s="4" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="C201" s="4" t="s">
         <v>15</v>
@@ -5348,7 +5390,7 @@
         <v>215</v>
       </c>
       <c r="B202" s="4" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="C202" s="4" t="s">
         <v>15</v>
@@ -5369,7 +5411,7 @@
         <v>216</v>
       </c>
       <c r="B203" s="4" t="s">
-        <v>217</v>
+        <v>230</v>
       </c>
       <c r="C203" s="4" t="s">
         <v>15</v>
@@ -5390,7 +5432,7 @@
         <v>217</v>
       </c>
       <c r="B204" s="4" t="s">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="C204" s="4" t="s">
         <v>15</v>
@@ -5411,7 +5453,7 @@
         <v>218</v>
       </c>
       <c r="B205" s="4" t="s">
-        <v>219</v>
+        <v>232</v>
       </c>
       <c r="C205" s="4" t="s">
         <v>15</v>
@@ -5432,7 +5474,7 @@
         <v>219</v>
       </c>
       <c r="B206" s="4" t="s">
-        <v>220</v>
+        <v>233</v>
       </c>
       <c r="C206" s="4" t="s">
         <v>15</v>
@@ -5453,7 +5495,7 @@
         <v>220</v>
       </c>
       <c r="B207" s="4" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
       <c r="C207" s="4" t="s">
         <v>15</v>
@@ -5474,7 +5516,7 @@
         <v>221</v>
       </c>
       <c r="B208" s="4" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="C208" s="4" t="s">
         <v>15</v>
@@ -5495,10 +5537,10 @@
         <v>222</v>
       </c>
       <c r="B209" s="4" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="C209" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D209" s="4" t="n">
         <v>1</v>
@@ -5516,20 +5558,20 @@
         <v>223</v>
       </c>
       <c r="B210" s="4" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="C210" s="4" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
       <c r="D210" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E210" s="5" t="n">
-        <v>69000</v>
+        <v>36000</v>
       </c>
       <c r="F210" s="5" t="n">
         <f aca="false">D210*E210</f>
-        <v>138000</v>
+        <v>72000</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5537,7 +5579,7 @@
         <v>224</v>
       </c>
       <c r="B211" s="4" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
       <c r="C211" s="4" t="s">
         <v>15</v>
@@ -5558,7 +5600,7 @@
         <v>225</v>
       </c>
       <c r="B212" s="4" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="C212" s="4" t="s">
         <v>11</v>
@@ -5579,7 +5621,7 @@
         <v>226</v>
       </c>
       <c r="B213" s="4" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="C213" s="4" t="s">
         <v>11</v>
@@ -5600,7 +5642,7 @@
         <v>227</v>
       </c>
       <c r="B214" s="4" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="C214" s="4" t="s">
         <v>11</v>
@@ -5621,7 +5663,7 @@
         <v>228</v>
       </c>
       <c r="B215" s="4" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="C215" s="4" t="s">
         <v>11</v>
@@ -5642,7 +5684,7 @@
         <v>229</v>
       </c>
       <c r="B216" s="4" t="s">
-        <v>230</v>
+        <v>243</v>
       </c>
       <c r="C216" s="4" t="s">
         <v>11</v>
@@ -5663,20 +5705,20 @@
         <v>230</v>
       </c>
       <c r="B217" s="4" t="s">
-        <v>231</v>
+        <v>244</v>
       </c>
       <c r="C217" s="4" t="s">
-        <v>15</v>
+        <v>245</v>
       </c>
       <c r="D217" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E217" s="5" t="n">
-        <v>9780</v>
+        <v>9750</v>
       </c>
       <c r="F217" s="5" t="n">
         <f aca="false">D217*E217</f>
-        <v>9780</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5684,20 +5726,20 @@
         <v>231</v>
       </c>
       <c r="B218" s="4" t="s">
-        <v>232</v>
+        <v>246</v>
       </c>
       <c r="C218" s="4" t="s">
-        <v>15</v>
+        <v>245</v>
       </c>
       <c r="D218" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E218" s="5" t="n">
-        <v>12650</v>
+        <v>8030</v>
       </c>
       <c r="F218" s="5" t="n">
         <f aca="false">D218*E218</f>
-        <v>12650</v>
+        <v>8030</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5705,20 +5747,20 @@
         <v>233</v>
       </c>
       <c r="B219" s="4" t="s">
-        <v>233</v>
+        <v>247</v>
       </c>
       <c r="C219" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D219" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E219" s="5" t="n">
-        <v>97750</v>
+        <v>52000</v>
       </c>
       <c r="F219" s="5" t="n">
         <f aca="false">D219*E219</f>
-        <v>195500</v>
+        <v>104000</v>
       </c>
     </row>
     <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5726,7 +5768,7 @@
         <v>234</v>
       </c>
       <c r="B220" s="4" t="s">
-        <v>234</v>
+        <v>248</v>
       </c>
       <c r="C220" s="4" t="s">
         <v>18</v>
@@ -5747,10 +5789,10 @@
         <v>235</v>
       </c>
       <c r="B221" s="4" t="s">
-        <v>235</v>
+        <v>249</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D221" s="4" t="n">
         <v>3</v>
@@ -5768,10 +5810,10 @@
         <v>236</v>
       </c>
       <c r="B222" s="4" t="s">
-        <v>236</v>
+        <v>250</v>
       </c>
       <c r="C222" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D222" s="4" t="n">
         <v>200</v>
@@ -5789,10 +5831,10 @@
         <v>237</v>
       </c>
       <c r="B223" s="4" t="s">
-        <v>237</v>
+        <v>251</v>
       </c>
       <c r="C223" s="4" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="D223" s="4" t="n">
         <v>24</v>
@@ -5810,10 +5852,10 @@
         <v>238</v>
       </c>
       <c r="B224" s="4" t="s">
-        <v>238</v>
+        <v>252</v>
       </c>
       <c r="C224" s="4" t="s">
-        <v>239</v>
+        <v>253</v>
       </c>
       <c r="D224" s="4" t="n">
         <v>6</v>
@@ -5831,10 +5873,10 @@
         <v>239</v>
       </c>
       <c r="B225" s="4" t="s">
-        <v>240</v>
+        <v>254</v>
       </c>
       <c r="C225" s="4" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D225" s="4" t="n">
         <v>50</v>
@@ -5852,7 +5894,7 @@
         <v>240</v>
       </c>
       <c r="B226" s="4" t="s">
-        <v>241</v>
+        <v>255</v>
       </c>
       <c r="C226" s="4" t="s">
         <v>15</v>
@@ -5870,11 +5912,11 @@
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E227" s="6" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="F227" s="7" t="n">
         <f aca="false">SUM(F5:F226)</f>
-        <v>13975036</v>
+        <v>13049175</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calibrated Licota/Yato/Bosch rates from brand dealer prices (UAE/PH) where no PK listing exists
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
@@ -1403,11 +1403,11 @@
         <v>4</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>24150</v>
+        <v>31050</v>
       </c>
       <c r="F14" s="5" t="n">
         <f aca="false">D14*E14</f>
-        <v>96600</v>
+        <v>124200</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1466,11 +1466,11 @@
         <v>4</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>34500</v>
+        <v>32200</v>
       </c>
       <c r="F17" s="5" t="n">
         <f aca="false">D17*E17</f>
-        <v>138000</v>
+        <v>128800</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1613,11 +1613,11 @@
         <v>3</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>1500</v>
+        <v>1440</v>
       </c>
       <c r="F24" s="5" t="n">
         <f aca="false">D24*E24</f>
-        <v>4500</v>
+        <v>4320</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1634,11 +1634,11 @@
         <v>3</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>1960</v>
+        <v>1840</v>
       </c>
       <c r="F25" s="5" t="n">
         <f aca="false">D25*E25</f>
-        <v>5880</v>
+        <v>5520</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1655,11 +1655,11 @@
         <v>3</v>
       </c>
       <c r="E26" s="5" t="n">
-        <v>2420</v>
+        <v>2300</v>
       </c>
       <c r="F26" s="5" t="n">
         <f aca="false">D26*E26</f>
-        <v>7260</v>
+        <v>6900</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1823,11 +1823,11 @@
         <v>3</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>5180</v>
+        <v>6670</v>
       </c>
       <c r="F34" s="5" t="n">
         <f aca="false">D34*E34</f>
-        <v>15540</v>
+        <v>20010</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1844,11 +1844,11 @@
         <v>3</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>6670</v>
+        <v>7820</v>
       </c>
       <c r="F35" s="5" t="n">
         <f aca="false">D35*E35</f>
-        <v>20010</v>
+        <v>23460</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1886,11 +1886,11 @@
         <v>2</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>17830</v>
+        <v>18400</v>
       </c>
       <c r="F37" s="5" t="n">
         <f aca="false">D37*E37</f>
-        <v>35660</v>
+        <v>36800</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1907,11 +1907,11 @@
         <v>2</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>33350</v>
+        <v>41400</v>
       </c>
       <c r="F38" s="5" t="n">
         <f aca="false">D38*E38</f>
-        <v>66700</v>
+        <v>82800</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1928,11 +1928,11 @@
         <v>3</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>6900</v>
+        <v>7250</v>
       </c>
       <c r="F39" s="5" t="n">
         <f aca="false">D39*E39</f>
-        <v>20700</v>
+        <v>21750</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1970,11 +1970,11 @@
         <v>3</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>8630</v>
+        <v>8050</v>
       </c>
       <c r="F41" s="5" t="n">
         <f aca="false">D41*E41</f>
-        <v>25890</v>
+        <v>24150</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2033,11 +2033,11 @@
         <v>3</v>
       </c>
       <c r="E44" s="5" t="n">
-        <v>161000</v>
+        <v>128700</v>
       </c>
       <c r="F44" s="5" t="n">
         <f aca="false">D44*E44</f>
-        <v>483000</v>
+        <v>386100</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2075,11 +2075,11 @@
         <v>4</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>2530</v>
+        <v>1840</v>
       </c>
       <c r="F46" s="5" t="n">
         <f aca="false">D46*E46</f>
-        <v>10120</v>
+        <v>7360</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2138,11 +2138,11 @@
         <v>3</v>
       </c>
       <c r="E49" s="5" t="n">
-        <v>18400</v>
+        <v>23000</v>
       </c>
       <c r="F49" s="5" t="n">
         <f aca="false">D49*E49</f>
-        <v>55200</v>
+        <v>69000</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2159,11 +2159,11 @@
         <v>2</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>27600</v>
+        <v>29900</v>
       </c>
       <c r="F50" s="5" t="n">
         <f aca="false">D50*E50</f>
-        <v>55200</v>
+        <v>59800</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2180,11 +2180,11 @@
         <v>1</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>32200</v>
+        <v>34500</v>
       </c>
       <c r="F51" s="5" t="n">
         <f aca="false">D51*E51</f>
-        <v>32200</v>
+        <v>34500</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2201,11 +2201,11 @@
         <v>1</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>43700</v>
+        <v>46000</v>
       </c>
       <c r="F52" s="5" t="n">
         <f aca="false">D52*E52</f>
-        <v>43700</v>
+        <v>46000</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2222,11 +2222,11 @@
         <v>1</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>51750</v>
+        <v>48300</v>
       </c>
       <c r="F53" s="5" t="n">
         <f aca="false">D53*E53</f>
-        <v>51750</v>
+        <v>48300</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2243,11 +2243,11 @@
         <v>2</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>23000</v>
+        <v>21850</v>
       </c>
       <c r="F54" s="5" t="n">
         <f aca="false">D54*E54</f>
-        <v>46000</v>
+        <v>43700</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2264,11 +2264,11 @@
         <v>1</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>34500</v>
+        <v>32200</v>
       </c>
       <c r="F55" s="5" t="n">
         <f aca="false">D55*E55</f>
-        <v>34500</v>
+        <v>32200</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2474,11 +2474,11 @@
         <v>1</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>12650</v>
+        <v>14380</v>
       </c>
       <c r="F65" s="5" t="n">
         <f aca="false">D65*E65</f>
-        <v>12650</v>
+        <v>14380</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3377,11 +3377,11 @@
         <v>3</v>
       </c>
       <c r="E108" s="5" t="n">
-        <v>5750</v>
+        <v>4830</v>
       </c>
       <c r="F108" s="5" t="n">
         <f aca="false">D108*E108</f>
-        <v>17250</v>
+        <v>14490</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5666,11 +5666,11 @@
         <v>1</v>
       </c>
       <c r="E217" s="5" t="n">
-        <v>9780</v>
+        <v>9750</v>
       </c>
       <c r="F217" s="5" t="n">
         <f aca="false">D217*E217</f>
-        <v>9780</v>
+        <v>9750</v>
       </c>
     </row>
     <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5687,11 +5687,11 @@
         <v>1</v>
       </c>
       <c r="E218" s="5" t="n">
-        <v>12650</v>
+        <v>12350</v>
       </c>
       <c r="F218" s="5" t="n">
         <f aca="false">D218*E218</f>
-        <v>12650</v>
+        <v>12350</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5868,7 +5868,7 @@
       </c>
       <c r="F227" s="7" t="n">
         <f aca="false">SUM(F5:F226)</f>
-        <v>15547300</v>
+        <v>15503200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use Pakistani-listed alternative brands where Licota/Yato/Dormer are not available online
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="247">
   <si>
     <t xml:space="preserve">Zidane Corporation - REVISED QUOTATION</t>
   </si>
@@ -49,7 +49,7 @@
     <t xml:space="preserve">STONE CUTTING DISC 4"</t>
   </si>
   <si>
-    <t xml:space="preserve">Bosch</t>
+    <t xml:space="preserve">Industrial</t>
   </si>
   <si>
     <t xml:space="preserve">STEEL NAIL 1-1/2" Taiwan</t>
@@ -76,9 +76,6 @@
     <t xml:space="preserve">SAFETY HELMET (WHITE)</t>
   </si>
   <si>
-    <t xml:space="preserve">Industrial</t>
-  </si>
-  <si>
     <t xml:space="preserve">SAFETY GOOGLES</t>
   </si>
   <si>
@@ -94,6 +91,9 @@
     <t xml:space="preserve">DOUBLE OPEN END WRENCH 6 TO 32 (12 PCS SET)</t>
   </si>
   <si>
+    <t xml:space="preserve">Harden</t>
+  </si>
+  <si>
     <t xml:space="preserve">DOUBLE OPEN END WRENCH 36X41</t>
   </si>
   <si>
@@ -103,6 +103,9 @@
     <t xml:space="preserve">COMBINATION WRENCH 8 TO 32 (14 PCS SET)</t>
   </si>
   <si>
+    <t xml:space="preserve">Tolsen</t>
+  </si>
+  <si>
     <t xml:space="preserve">SOCKET SET (113PCS) 1/4" &amp; 1/2"</t>
   </si>
   <si>
@@ -154,6 +157,9 @@
     <t xml:space="preserve">PIPE WRENCH SIZE 10"</t>
   </si>
   <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
     <t xml:space="preserve">PIPE WRENCH SIZE 12"</t>
   </si>
   <si>
@@ -247,6 +253,9 @@
     <t xml:space="preserve">STEEL MEASURMENT TAPE 50M</t>
   </si>
   <si>
+    <t xml:space="preserve">Ingco</t>
+  </si>
+  <si>
     <t xml:space="preserve">ALIGNING PRY BAR DIA 5/8" X 18" LENGTH</t>
   </si>
   <si>
@@ -538,6 +547,9 @@
     <t xml:space="preserve">ANCHOR BOLT 10X110</t>
   </si>
   <si>
+    <t xml:space="preserve">SMT</t>
+  </si>
+  <si>
     <t xml:space="preserve">ANCHOR BOLT 12X120</t>
   </si>
   <si>
@@ -646,6 +658,9 @@
     <t xml:space="preserve">END MILL CUTTER SIZE 12MM</t>
   </si>
   <si>
+    <t xml:space="preserve">HSS</t>
+  </si>
+  <si>
     <t xml:space="preserve">END MILL CUTTER SIZE 16MM</t>
   </si>
   <si>
@@ -710,6 +725,9 @@
   </si>
   <si>
     <t xml:space="preserve">HYDRAULIC JACK 3 TON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ronix</t>
   </si>
   <si>
     <t xml:space="preserve">HYDRAULIC JACK 5 TON</t>
@@ -1313,7 +1331,7 @@
         <v>17</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>6</v>
@@ -1331,10 +1349,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D11" s="4" t="n">
         <v>24</v>
@@ -1352,10 +1370,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="D12" s="4" t="n">
         <v>3</v>
@@ -1373,10 +1391,10 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>4</v>
@@ -1394,20 +1412,20 @@
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>23</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>31050</v>
+        <v>15600</v>
       </c>
       <c r="F14" s="5" t="n">
         <f aca="false">D14*E14</f>
-        <v>124200</v>
+        <v>62400</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1418,7 +1436,7 @@
         <v>24</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>3</v>
@@ -1439,7 +1457,7 @@
         <v>25</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>3</v>
@@ -1460,17 +1478,17 @@
         <v>26</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D17" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>32200</v>
+        <v>15900</v>
       </c>
       <c r="F17" s="5" t="n">
         <f aca="false">D17*E17</f>
-        <v>128800</v>
+        <v>63600</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1478,10 +1496,10 @@
         <v>14</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D18" s="4" t="n">
         <v>4</v>
@@ -1499,10 +1517,10 @@
         <v>15</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D19" s="4" t="n">
         <v>4</v>
@@ -1520,20 +1538,20 @@
         <v>16</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>4</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>18400</v>
+        <v>8450</v>
       </c>
       <c r="F20" s="5" t="n">
         <f aca="false">D20*E20</f>
-        <v>73600</v>
+        <v>33800</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1541,10 +1559,10 @@
         <v>17</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>4</v>
@@ -1562,10 +1580,10 @@
         <v>18</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D22" s="4" t="n">
         <v>4</v>
@@ -1583,10 +1601,10 @@
         <v>19</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>4</v>
@@ -1604,10 +1622,10 @@
         <v>20</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D24" s="4" t="n">
         <v>3</v>
@@ -1625,10 +1643,10 @@
         <v>21</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D25" s="4" t="n">
         <v>3</v>
@@ -1646,10 +1664,10 @@
         <v>22</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D26" s="4" t="n">
         <v>3</v>
@@ -1667,10 +1685,10 @@
         <v>23</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D27" s="4" t="n">
         <v>4</v>
@@ -1688,10 +1706,10 @@
         <v>24</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D28" s="4" t="n">
         <v>4</v>
@@ -1709,10 +1727,10 @@
         <v>25</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D29" s="4" t="n">
         <v>4</v>
@@ -1730,10 +1748,10 @@
         <v>26</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D30" s="4" t="n">
         <v>4</v>
@@ -1751,10 +1769,10 @@
         <v>27</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D31" s="4" t="n">
         <v>4</v>
@@ -1772,10 +1790,10 @@
         <v>28</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D32" s="4" t="n">
         <v>3</v>
@@ -1793,10 +1811,10 @@
         <v>30</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D33" s="4" t="n">
         <v>4</v>
@@ -1814,20 +1832,20 @@
         <v>31</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="D34" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E34" s="5" t="n">
-        <v>6670</v>
+        <v>2210</v>
       </c>
       <c r="F34" s="5" t="n">
         <f aca="false">D34*E34</f>
-        <v>20010</v>
+        <v>6630</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1835,20 +1853,20 @@
         <v>32</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D35" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E35" s="5" t="n">
-        <v>7820</v>
+        <v>3280</v>
       </c>
       <c r="F35" s="5" t="n">
         <f aca="false">D35*E35</f>
-        <v>23460</v>
+        <v>9840</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1856,10 +1874,10 @@
         <v>33</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D36" s="4" t="n">
         <v>3</v>
@@ -1877,20 +1895,20 @@
         <v>34</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D37" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>18400</v>
+        <v>7540</v>
       </c>
       <c r="F37" s="5" t="n">
         <f aca="false">D37*E37</f>
-        <v>36800</v>
+        <v>15080</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1898,20 +1916,20 @@
         <v>35</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="D38" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E38" s="5" t="n">
-        <v>41400</v>
+        <v>12870</v>
       </c>
       <c r="F38" s="5" t="n">
         <f aca="false">D38*E38</f>
-        <v>82800</v>
+        <v>25740</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1919,20 +1937,20 @@
         <v>36</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="D39" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E39" s="5" t="n">
-        <v>7250</v>
+        <v>2300</v>
       </c>
       <c r="F39" s="5" t="n">
         <f aca="false">D39*E39</f>
-        <v>21750</v>
+        <v>6900</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1940,20 +1958,20 @@
         <v>37</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D40" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E40" s="5" t="n">
-        <v>10930</v>
+        <v>4550</v>
       </c>
       <c r="F40" s="5" t="n">
         <f aca="false">D40*E40</f>
-        <v>32790</v>
+        <v>13650</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1961,20 +1979,20 @@
         <v>38</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D41" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>8050</v>
+        <v>3310</v>
       </c>
       <c r="F41" s="5" t="n">
         <f aca="false">D41*E41</f>
-        <v>24150</v>
+        <v>9930</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1982,10 +2000,10 @@
         <v>39</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D42" s="4" t="n">
         <v>3</v>
@@ -2003,10 +2021,10 @@
         <v>40</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D43" s="4" t="n">
         <v>3</v>
@@ -2024,10 +2042,10 @@
         <v>41</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D44" s="4" t="n">
         <v>3</v>
@@ -2045,10 +2063,10 @@
         <v>42</v>
       </c>
       <c r="B45" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C45" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="D45" s="4" t="n">
         <v>2</v>
@@ -2066,10 +2084,10 @@
         <v>43</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D46" s="4" t="n">
         <v>4</v>
@@ -2087,10 +2105,10 @@
         <v>44</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D47" s="4" t="n">
         <v>4</v>
@@ -2108,10 +2126,10 @@
         <v>45</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D48" s="4" t="n">
         <v>4</v>
@@ -2129,10 +2147,10 @@
         <v>47</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D49" s="4" t="n">
         <v>3</v>
@@ -2150,10 +2168,10 @@
         <v>48</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D50" s="4" t="n">
         <v>2</v>
@@ -2171,10 +2189,10 @@
         <v>49</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D51" s="4" t="n">
         <v>1</v>
@@ -2192,10 +2210,10 @@
         <v>50</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D52" s="4" t="n">
         <v>1</v>
@@ -2213,10 +2231,10 @@
         <v>51</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D53" s="4" t="n">
         <v>1</v>
@@ -2234,20 +2252,20 @@
         <v>52</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="D54" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>21850</v>
+        <v>11480</v>
       </c>
       <c r="F54" s="5" t="n">
         <f aca="false">D54*E54</f>
-        <v>43700</v>
+        <v>22960</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2255,20 +2273,20 @@
         <v>53</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>21</v>
+        <v>60</v>
       </c>
       <c r="D55" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E55" s="5" t="n">
-        <v>32200</v>
+        <v>23400</v>
       </c>
       <c r="F55" s="5" t="n">
         <f aca="false">D55*E55</f>
-        <v>32200</v>
+        <v>23400</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2276,10 +2294,10 @@
         <v>54</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D56" s="4" t="n">
         <v>2</v>
@@ -2297,10 +2315,10 @@
         <v>55</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D57" s="4" t="n">
         <v>2</v>
@@ -2318,10 +2336,10 @@
         <v>56</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D58" s="4" t="n">
         <v>1</v>
@@ -2339,10 +2357,10 @@
         <v>57</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D59" s="4" t="n">
         <v>4</v>
@@ -2360,10 +2378,10 @@
         <v>58</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D60" s="4" t="n">
         <v>12</v>
@@ -2381,10 +2399,10 @@
         <v>59</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D61" s="4" t="n">
         <v>12</v>
@@ -2402,20 +2420,20 @@
         <v>60</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D62" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>13800</v>
+        <v>9100</v>
       </c>
       <c r="F62" s="5" t="n">
         <f aca="false">D62*E62</f>
-        <v>27600</v>
+        <v>18200</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2423,20 +2441,20 @@
         <v>61</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="D63" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>8630</v>
+        <v>6810</v>
       </c>
       <c r="F63" s="5" t="n">
         <f aca="false">D63*E63</f>
-        <v>17260</v>
+        <v>13620</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2444,20 +2462,20 @@
         <v>62</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="D64" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>4600</v>
+        <v>4020</v>
       </c>
       <c r="F64" s="5" t="n">
         <f aca="false">D64*E64</f>
-        <v>13800</v>
+        <v>12060</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2465,20 +2483,20 @@
         <v>63</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="D65" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>14380</v>
+        <v>5551</v>
       </c>
       <c r="F65" s="5" t="n">
         <f aca="false">D65*E65</f>
-        <v>14380</v>
+        <v>5551</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2486,10 +2504,10 @@
         <v>64</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D66" s="4" t="n">
         <v>3</v>
@@ -2507,10 +2525,10 @@
         <v>65</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D67" s="4" t="n">
         <v>3</v>
@@ -2528,10 +2546,10 @@
         <v>66</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D68" s="4" t="n">
         <v>2</v>
@@ -2549,10 +2567,10 @@
         <v>67</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D69" s="4" t="n">
         <v>2</v>
@@ -2570,10 +2588,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D70" s="4" t="n">
         <v>2</v>
@@ -2591,10 +2609,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D71" s="4" t="n">
         <v>1</v>
@@ -2612,20 +2630,20 @@
         <v>71</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D72" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E72" s="5" t="n">
-        <v>1380</v>
+        <v>1150</v>
       </c>
       <c r="F72" s="5" t="n">
         <f aca="false">D72*E72</f>
-        <v>1380</v>
+        <v>1150</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2633,20 +2651,20 @@
         <v>73</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
       <c r="D73" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E73" s="5" t="n">
-        <v>63250</v>
+        <v>29950</v>
       </c>
       <c r="F73" s="5" t="n">
         <f aca="false">D73*E73</f>
-        <v>63250</v>
+        <v>29950</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2654,7 +2672,7 @@
         <v>74</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>15</v>
@@ -2675,7 +2693,7 @@
         <v>75</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>15</v>
@@ -2696,7 +2714,7 @@
         <v>76</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>15</v>
@@ -2717,7 +2735,7 @@
         <v>77</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>15</v>
@@ -2738,7 +2756,7 @@
         <v>78</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>15</v>
@@ -2759,7 +2777,7 @@
         <v>79</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>15</v>
@@ -2780,7 +2798,7 @@
         <v>80</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>15</v>
@@ -2801,7 +2819,7 @@
         <v>81</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>15</v>
@@ -2822,7 +2840,7 @@
         <v>82</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>15</v>
@@ -2843,7 +2861,7 @@
         <v>83</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C83" s="4" t="s">
         <v>15</v>
@@ -2864,7 +2882,7 @@
         <v>84</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>15</v>
@@ -2885,7 +2903,7 @@
         <v>85</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C85" s="4" t="s">
         <v>15</v>
@@ -2906,7 +2924,7 @@
         <v>86</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>15</v>
@@ -2927,7 +2945,7 @@
         <v>87</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>15</v>
@@ -2948,10 +2966,10 @@
         <v>88</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D88" s="4" t="n">
         <v>2</v>
@@ -2969,10 +2987,10 @@
         <v>89</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D89" s="4" t="n">
         <v>2</v>
@@ -2990,10 +3008,10 @@
         <v>90</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D90" s="4" t="n">
         <v>2</v>
@@ -3011,10 +3029,10 @@
         <v>91</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D91" s="4" t="n">
         <v>2</v>
@@ -3032,10 +3050,10 @@
         <v>92</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D92" s="4" t="n">
         <v>2</v>
@@ -3053,10 +3071,10 @@
         <v>93</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D93" s="4" t="n">
         <v>2</v>
@@ -3074,10 +3092,10 @@
         <v>94</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D94" s="4" t="n">
         <v>3</v>
@@ -3095,10 +3113,10 @@
         <v>95</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D95" s="4" t="n">
         <v>3</v>
@@ -3116,10 +3134,10 @@
         <v>96</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D96" s="4" t="n">
         <v>2</v>
@@ -3137,10 +3155,10 @@
         <v>97</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D97" s="4" t="n">
         <v>2</v>
@@ -3158,7 +3176,7 @@
         <v>98</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C98" s="4" t="s">
         <v>15</v>
@@ -3179,7 +3197,7 @@
         <v>99</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>15</v>
@@ -3200,7 +3218,7 @@
         <v>100</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C100" s="4" t="s">
         <v>15</v>
@@ -3221,7 +3239,7 @@
         <v>101</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C101" s="4" t="s">
         <v>15</v>
@@ -3242,7 +3260,7 @@
         <v>102</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C102" s="4" t="s">
         <v>15</v>
@@ -3263,10 +3281,10 @@
         <v>103</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D103" s="4" t="n">
         <v>12</v>
@@ -3284,10 +3302,10 @@
         <v>104</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D104" s="4" t="n">
         <v>4</v>
@@ -3305,10 +3323,10 @@
         <v>105</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D105" s="4" t="n">
         <v>12</v>
@@ -3326,10 +3344,10 @@
         <v>106</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D106" s="4" t="n">
         <v>6</v>
@@ -3347,10 +3365,10 @@
         <v>107</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D107" s="4" t="n">
         <v>6</v>
@@ -3368,20 +3386,20 @@
         <v>108</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D108" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E108" s="5" t="n">
-        <v>4830</v>
+        <v>4550</v>
       </c>
       <c r="F108" s="5" t="n">
         <f aca="false">D108*E108</f>
-        <v>14490</v>
+        <v>13650</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3389,10 +3407,10 @@
         <v>109</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D109" s="4" t="n">
         <v>6</v>
@@ -3410,20 +3428,20 @@
         <v>110</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D110" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E110" s="5" t="n">
-        <v>3220</v>
+        <v>1160</v>
       </c>
       <c r="F110" s="5" t="n">
         <f aca="false">D110*E110</f>
-        <v>9660</v>
+        <v>3480</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3431,20 +3449,20 @@
         <v>111</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>83</v>
+        <v>23</v>
       </c>
       <c r="D111" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E111" s="5" t="n">
-        <v>6330</v>
+        <v>3590</v>
       </c>
       <c r="F111" s="5" t="n">
         <f aca="false">D111*E111</f>
-        <v>18990</v>
+        <v>10770</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3452,20 +3470,20 @@
         <v>112</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D112" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E112" s="5" t="n">
-        <v>13800</v>
+        <v>12350</v>
       </c>
       <c r="F112" s="5" t="n">
         <f aca="false">D112*E112</f>
-        <v>27600</v>
+        <v>24700</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3473,20 +3491,20 @@
         <v>113</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D113" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E113" s="5" t="n">
-        <v>1560</v>
+        <v>1840</v>
       </c>
       <c r="F113" s="5" t="n">
         <f aca="false">D113*E113</f>
-        <v>4680</v>
+        <v>5520</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3494,10 +3512,10 @@
         <v>114</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D114" s="4" t="n">
         <v>3</v>
@@ -3515,10 +3533,10 @@
         <v>115</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D115" s="4" t="n">
         <v>2</v>
@@ -3536,10 +3554,10 @@
         <v>116</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D116" s="4" t="n">
         <v>2</v>
@@ -3557,10 +3575,10 @@
         <v>117</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D117" s="4" t="n">
         <v>15</v>
@@ -3578,10 +3596,10 @@
         <v>118</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D118" s="4" t="n">
         <v>15</v>
@@ -3599,10 +3617,10 @@
         <v>119</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D119" s="4" t="n">
         <v>2</v>
@@ -3620,10 +3638,10 @@
         <v>120</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D120" s="4" t="n">
         <v>6</v>
@@ -3641,10 +3659,10 @@
         <v>121</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D121" s="4" t="n">
         <v>6</v>
@@ -3662,20 +3680,20 @@
         <v>122</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D122" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E122" s="5" t="n">
-        <v>379500</v>
+        <v>170100</v>
       </c>
       <c r="F122" s="5" t="n">
         <f aca="false">D122*E122</f>
-        <v>379500</v>
+        <v>170100</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3683,10 +3701,10 @@
         <v>123</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D123" s="4" t="n">
         <v>2</v>
@@ -3704,10 +3722,10 @@
         <v>124</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D124" s="4" t="n">
         <v>2</v>
@@ -3725,10 +3743,10 @@
         <v>125</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D125" s="4" t="n">
         <v>12</v>
@@ -3746,10 +3764,10 @@
         <v>126</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D126" s="4" t="n">
         <v>12</v>
@@ -3767,10 +3785,10 @@
         <v>127</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D127" s="4" t="n">
         <v>6</v>
@@ -3788,10 +3806,10 @@
         <v>128</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D128" s="4" t="n">
         <v>6</v>
@@ -3809,10 +3827,10 @@
         <v>129</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D129" s="4" t="n">
         <v>6</v>
@@ -3830,10 +3848,10 @@
         <v>130</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D130" s="4" t="n">
         <v>6</v>
@@ -3851,10 +3869,10 @@
         <v>131</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D131" s="4" t="n">
         <v>2</v>
@@ -3872,10 +3890,10 @@
         <v>132</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D132" s="4" t="n">
         <v>10</v>
@@ -3893,10 +3911,10 @@
         <v>133</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D133" s="4" t="n">
         <v>6</v>
@@ -3914,10 +3932,10 @@
         <v>134</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D134" s="4" t="n">
         <v>6</v>
@@ -3935,10 +3953,10 @@
         <v>135</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D135" s="4" t="n">
         <v>6</v>
@@ -3956,10 +3974,10 @@
         <v>136</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C136" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D136" s="4" t="n">
         <v>500</v>
@@ -3977,10 +3995,10 @@
         <v>138</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D137" s="4" t="n">
         <v>24</v>
@@ -3998,10 +4016,10 @@
         <v>139</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D138" s="4" t="n">
         <v>24</v>
@@ -4019,10 +4037,10 @@
         <v>140</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D139" s="4" t="n">
         <v>24</v>
@@ -4040,10 +4058,10 @@
         <v>142</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D140" s="4" t="n">
         <v>3</v>
@@ -4061,10 +4079,10 @@
         <v>143</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D141" s="4" t="n">
         <v>3</v>
@@ -4082,10 +4100,10 @@
         <v>144</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D142" s="4" t="n">
         <v>3</v>
@@ -4103,10 +4121,10 @@
         <v>145</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D143" s="4" t="n">
         <v>500</v>
@@ -4124,10 +4142,10 @@
         <v>146</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C144" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D144" s="4" t="n">
         <v>1</v>
@@ -4145,10 +4163,10 @@
         <v>147</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D145" s="4" t="n">
         <v>1</v>
@@ -4166,20 +4184,20 @@
         <v>148</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C146" s="4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D146" s="4" t="n">
         <v>12</v>
       </c>
       <c r="E146" s="5" t="n">
-        <v>1380</v>
+        <v>490</v>
       </c>
       <c r="F146" s="5" t="n">
         <f aca="false">D146*E146</f>
-        <v>16560</v>
+        <v>5880</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4187,10 +4205,10 @@
         <v>149</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D147" s="4" t="n">
         <v>100</v>
@@ -4208,10 +4226,10 @@
         <v>150</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C148" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D148" s="4" t="n">
         <v>100</v>
@@ -4229,10 +4247,10 @@
         <v>151</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D149" s="4" t="n">
         <v>100</v>
@@ -4250,10 +4268,10 @@
         <v>152</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C150" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D150" s="4" t="n">
         <v>24</v>
@@ -4271,10 +4289,10 @@
         <v>153</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D151" s="4" t="n">
         <v>24</v>
@@ -4292,10 +4310,10 @@
         <v>154</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D152" s="4" t="n">
         <v>12</v>
@@ -4313,10 +4331,10 @@
         <v>155</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D153" s="4" t="n">
         <v>50</v>
@@ -4334,10 +4352,10 @@
         <v>156</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D154" s="4" t="n">
         <v>30</v>
@@ -4355,10 +4373,10 @@
         <v>157</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D155" s="4" t="n">
         <v>30</v>
@@ -4376,10 +4394,10 @@
         <v>158</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D156" s="4" t="n">
         <v>12</v>
@@ -4397,10 +4415,10 @@
         <v>159</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D157" s="4" t="n">
         <v>100</v>
@@ -4418,20 +4436,20 @@
         <v>160</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>155</v>
+        <v>175</v>
       </c>
       <c r="D158" s="4" t="n">
         <v>150</v>
       </c>
       <c r="E158" s="5" t="n">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F158" s="5" t="n">
         <f aca="false">D158*E158</f>
-        <v>18000</v>
+        <v>17550</v>
       </c>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4439,10 +4457,10 @@
         <v>161</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D159" s="4" t="n">
         <v>150</v>
@@ -4460,10 +4478,10 @@
         <v>162</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D160" s="4" t="n">
         <v>150</v>
@@ -4481,10 +4499,10 @@
         <v>164</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D161" s="4" t="n">
         <v>40</v>
@@ -4502,10 +4520,10 @@
         <v>165</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D162" s="4" t="n">
         <v>40</v>
@@ -4523,10 +4541,10 @@
         <v>166</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D163" s="4" t="n">
         <v>20</v>
@@ -4544,10 +4562,10 @@
         <v>167</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="C164" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D164" s="4" t="n">
         <v>40</v>
@@ -4565,10 +4583,10 @@
         <v>168</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="C165" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D165" s="4" t="n">
         <v>20</v>
@@ -4586,20 +4604,20 @@
         <v>177</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C166" s="4" t="s">
-        <v>155</v>
+        <v>77</v>
       </c>
       <c r="D166" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E166" s="5" t="n">
-        <v>5850</v>
+        <v>1070</v>
       </c>
       <c r="F166" s="5" t="n">
         <f aca="false">D166*E166</f>
-        <v>17550</v>
+        <v>3210</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4607,7 +4625,7 @@
         <v>179</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="C167" s="4" t="s">
         <v>15</v>
@@ -4628,7 +4646,7 @@
         <v>180</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C168" s="4" t="s">
         <v>15</v>
@@ -4649,7 +4667,7 @@
         <v>181</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="C169" s="4" t="s">
         <v>15</v>
@@ -4670,7 +4688,7 @@
         <v>182</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="C170" s="4" t="s">
         <v>15</v>
@@ -4691,10 +4709,10 @@
         <v>183</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="C171" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D171" s="4" t="n">
         <v>3</v>
@@ -4712,10 +4730,10 @@
         <v>184</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C172" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D172" s="4" t="n">
         <v>3</v>
@@ -4733,10 +4751,10 @@
         <v>185</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="C173" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D173" s="4" t="n">
         <v>3</v>
@@ -4754,10 +4772,10 @@
         <v>186</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="C174" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D174" s="4" t="n">
         <v>3</v>
@@ -4775,10 +4793,10 @@
         <v>187</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C175" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D175" s="4" t="n">
         <v>2</v>
@@ -4796,10 +4814,10 @@
         <v>188</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="C176" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D176" s="4" t="n">
         <v>1</v>
@@ -4817,10 +4835,10 @@
         <v>189</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D177" s="4" t="n">
         <v>1</v>
@@ -4838,10 +4856,10 @@
         <v>190</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D178" s="4" t="n">
         <v>2</v>
@@ -4859,10 +4877,10 @@
         <v>191</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D179" s="4" t="n">
         <v>2</v>
@@ -4880,7 +4898,7 @@
         <v>192</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="C180" s="4" t="s">
         <v>11</v>
@@ -4901,7 +4919,7 @@
         <v>193</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="C181" s="4" t="s">
         <v>11</v>
@@ -4922,7 +4940,7 @@
         <v>194</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C182" s="4" t="s">
         <v>11</v>
@@ -4943,7 +4961,7 @@
         <v>195</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="C183" s="4" t="s">
         <v>11</v>
@@ -4964,10 +4982,10 @@
         <v>196</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="C184" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D184" s="4" t="n">
         <v>2</v>
@@ -4985,10 +5003,10 @@
         <v>197</v>
       </c>
       <c r="B185" s="4" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D185" s="4" t="n">
         <v>1</v>
@@ -5006,10 +5024,10 @@
         <v>198</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="C186" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D186" s="4" t="n">
         <v>1</v>
@@ -5027,10 +5045,10 @@
         <v>199</v>
       </c>
       <c r="B187" s="4" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D187" s="4" t="n">
         <v>1</v>
@@ -5048,10 +5066,10 @@
         <v>200</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C188" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D188" s="4" t="n">
         <v>1</v>
@@ -5069,10 +5087,10 @@
         <v>201</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="C189" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D189" s="4" t="n">
         <v>1</v>
@@ -5090,10 +5108,10 @@
         <v>202</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="C190" s="4" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="D190" s="4" t="n">
         <v>2</v>
@@ -5111,7 +5129,7 @@
         <v>204</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="C191" s="4" t="s">
         <v>15</v>
@@ -5132,7 +5150,7 @@
         <v>205</v>
       </c>
       <c r="B192" s="4" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C192" s="4" t="s">
         <v>15</v>
@@ -5153,7 +5171,7 @@
         <v>206</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="C193" s="4" t="s">
         <v>15</v>
@@ -5174,7 +5192,7 @@
         <v>207</v>
       </c>
       <c r="B194" s="4" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="C194" s="4" t="s">
         <v>15</v>
@@ -5195,20 +5213,20 @@
         <v>208</v>
       </c>
       <c r="B195" s="4" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="C195" s="4" t="s">
-        <v>15</v>
+        <v>212</v>
       </c>
       <c r="D195" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E195" s="5" t="n">
-        <v>16510</v>
+        <v>3340</v>
       </c>
       <c r="F195" s="5" t="n">
         <f aca="false">D195*E195</f>
-        <v>49530</v>
+        <v>10020</v>
       </c>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5216,7 +5234,7 @@
         <v>209</v>
       </c>
       <c r="B196" s="4" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C196" s="4" t="s">
         <v>15</v>
@@ -5237,7 +5255,7 @@
         <v>210</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C197" s="4" t="s">
         <v>15</v>
@@ -5258,7 +5276,7 @@
         <v>211</v>
       </c>
       <c r="B198" s="4" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C198" s="4" t="s">
         <v>15</v>
@@ -5279,7 +5297,7 @@
         <v>212</v>
       </c>
       <c r="B199" s="4" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C199" s="4" t="s">
         <v>15</v>
@@ -5300,10 +5318,10 @@
         <v>213</v>
       </c>
       <c r="B200" s="4" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D200" s="4" t="n">
         <v>2</v>
@@ -5321,10 +5339,10 @@
         <v>214</v>
       </c>
       <c r="B201" s="4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D201" s="4" t="n">
         <v>2</v>
@@ -5342,10 +5360,10 @@
         <v>215</v>
       </c>
       <c r="B202" s="4" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="C202" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D202" s="4" t="n">
         <v>2</v>
@@ -5363,10 +5381,10 @@
         <v>216</v>
       </c>
       <c r="B203" s="4" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D203" s="4" t="n">
         <v>2</v>
@@ -5384,10 +5402,10 @@
         <v>217</v>
       </c>
       <c r="B204" s="4" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C204" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D204" s="4" t="n">
         <v>2</v>
@@ -5405,10 +5423,10 @@
         <v>218</v>
       </c>
       <c r="B205" s="4" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C205" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D205" s="4" t="n">
         <v>2</v>
@@ -5426,10 +5444,10 @@
         <v>219</v>
       </c>
       <c r="B206" s="4" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="C206" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D206" s="4" t="n">
         <v>1</v>
@@ -5447,10 +5465,10 @@
         <v>220</v>
       </c>
       <c r="B207" s="4" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C207" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D207" s="4" t="n">
         <v>1</v>
@@ -5468,10 +5486,10 @@
         <v>221</v>
       </c>
       <c r="B208" s="4" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="C208" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D208" s="4" t="n">
         <v>1</v>
@@ -5489,10 +5507,10 @@
         <v>222</v>
       </c>
       <c r="B209" s="4" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="C209" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D209" s="4" t="n">
         <v>1</v>
@@ -5510,20 +5528,20 @@
         <v>223</v>
       </c>
       <c r="B210" s="4" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C210" s="4" t="s">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="D210" s="4" t="n">
         <v>2</v>
       </c>
       <c r="E210" s="5" t="n">
-        <v>69000</v>
+        <v>36000</v>
       </c>
       <c r="F210" s="5" t="n">
         <f aca="false">D210*E210</f>
-        <v>138000</v>
+        <v>72000</v>
       </c>
     </row>
     <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5531,10 +5549,10 @@
         <v>224</v>
       </c>
       <c r="B211" s="4" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="C211" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D211" s="4" t="n">
         <v>2</v>
@@ -5552,7 +5570,7 @@
         <v>225</v>
       </c>
       <c r="B212" s="4" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="C212" s="4" t="s">
         <v>15</v>
@@ -5573,7 +5591,7 @@
         <v>226</v>
       </c>
       <c r="B213" s="4" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="C213" s="4" t="s">
         <v>15</v>
@@ -5594,7 +5612,7 @@
         <v>227</v>
       </c>
       <c r="B214" s="4" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="C214" s="4" t="s">
         <v>15</v>
@@ -5615,7 +5633,7 @@
         <v>228</v>
       </c>
       <c r="B215" s="4" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C215" s="4" t="s">
         <v>15</v>
@@ -5636,7 +5654,7 @@
         <v>229</v>
       </c>
       <c r="B216" s="4" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="C216" s="4" t="s">
         <v>15</v>
@@ -5657,10 +5675,10 @@
         <v>230</v>
       </c>
       <c r="B217" s="4" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="C217" s="4" t="s">
-        <v>58</v>
+        <v>235</v>
       </c>
       <c r="D217" s="4" t="n">
         <v>1</v>
@@ -5678,20 +5696,20 @@
         <v>231</v>
       </c>
       <c r="B218" s="4" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="C218" s="4" t="s">
-        <v>58</v>
+        <v>235</v>
       </c>
       <c r="D218" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E218" s="5" t="n">
-        <v>12350</v>
+        <v>8030</v>
       </c>
       <c r="F218" s="5" t="n">
         <f aca="false">D218*E218</f>
-        <v>12350</v>
+        <v>8030</v>
       </c>
     </row>
     <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5699,10 +5717,10 @@
         <v>233</v>
       </c>
       <c r="B219" s="4" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="C219" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D219" s="4" t="n">
         <v>2</v>
@@ -5720,10 +5738,10 @@
         <v>234</v>
       </c>
       <c r="B220" s="4" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="C220" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D220" s="4" t="n">
         <v>3</v>
@@ -5741,20 +5759,20 @@
         <v>235</v>
       </c>
       <c r="B221" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="C221" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D221" s="4" t="n">
         <v>3</v>
       </c>
       <c r="E221" s="5" t="n">
-        <v>2860</v>
+        <v>680</v>
       </c>
       <c r="F221" s="5" t="n">
         <f aca="false">D221*E221</f>
-        <v>8580</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5762,10 +5780,10 @@
         <v>236</v>
       </c>
       <c r="B222" s="4" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="C222" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D222" s="4" t="n">
         <v>200</v>
@@ -5783,20 +5801,20 @@
         <v>237</v>
       </c>
       <c r="B223" s="4" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="C223" s="4" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="D223" s="4" t="n">
         <v>24</v>
       </c>
       <c r="E223" s="5" t="n">
-        <v>845</v>
+        <v>200</v>
       </c>
       <c r="F223" s="5" t="n">
         <f aca="false">D223*E223</f>
-        <v>20280</v>
+        <v>4800</v>
       </c>
     </row>
     <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5804,10 +5822,10 @@
         <v>238</v>
       </c>
       <c r="B224" s="4" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="C224" s="4" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="D224" s="4" t="n">
         <v>6</v>
@@ -5825,10 +5843,10 @@
         <v>239</v>
       </c>
       <c r="B225" s="4" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="C225" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D225" s="4" t="n">
         <v>50</v>
@@ -5846,7 +5864,7 @@
         <v>240</v>
       </c>
       <c r="B226" s="4" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="C226" s="4" t="s">
         <v>15</v>
@@ -5864,11 +5882,11 @@
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E227" s="6" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="F227" s="7" t="n">
         <f aca="false">SUM(F5:F226)</f>
-        <v>15503200</v>
+        <v>14711711</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Quotation: mark foreign-sourced lines as '<brand> / Equivalent'; fit 46 rows per PDF page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="453" uniqueCount="253">
   <si>
     <t xml:space="preserve">Zidane Corporation - REVISED QUOTATION</t>
   </si>
@@ -55,19 +55,19 @@
     <t xml:space="preserve">STEEL NAIL 1-1/2" Taiwan</t>
   </si>
   <si>
-    <t xml:space="preserve">Taiwan</t>
+    <t xml:space="preserve">Taiwan / Equivalent</t>
   </si>
   <si>
     <t xml:space="preserve">MECHANICAL JACK 5 TON (Japan or Germany)</t>
   </si>
   <si>
-    <t xml:space="preserve">JET (Taiwan)</t>
+    <t xml:space="preserve">JET (Taiwan) / Equivalent</t>
   </si>
   <si>
     <t xml:space="preserve">DRILL BIT 08 MM (Yato or any Good brand taiwan)</t>
   </si>
   <si>
-    <t xml:space="preserve">Dormer</t>
+    <t xml:space="preserve">Dormer / Equivalent</t>
   </si>
   <si>
     <t xml:space="preserve">MECHANICAL JACK 03 TONS (Japan or germany)</t>
@@ -127,87 +127,96 @@
     <t xml:space="preserve">ALLEN HEX KEY 12MM</t>
   </si>
   <si>
+    <t xml:space="preserve">Licota / Equivalent</t>
+  </si>
+  <si>
     <t xml:space="preserve">ALLEN (HEX) KEY 14MM</t>
   </si>
   <si>
+    <t xml:space="preserve">Yato / Equivalent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALLEN (HEX) KEY 16MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER INTERNAL STRAIGHT 175MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER INTERNAL BENT 175MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL STRAIGHT 175MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL BENT 175MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHISEL SET (05 PCS SET)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIPE WRENCH SIZE 10"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIPE WRENCH SIZE 12"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIPE WRENCH SIZE 18"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIPE WRENCH SIZE 24"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PIPE WRENCH SIZE 36"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SLEDGE HAMMER 3 LBS WITH FIBREGLASS HANDLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOFT FACE DEAD BLOW HAMMER 50MM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VICE GRIP PLIER 08"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORDLESS IMPACT WRENCH 185NM (Bosch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bosch Professional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORDLESS IMPACT WRENCH 350N (Bosch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bosch Professional / Equivalent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CORDLESS IMPACT WRENCH 1000N (Bosch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DeWalt / Equivalent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLAT FILE 12"</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yato</t>
   </si>
   <si>
-    <t xml:space="preserve">ALLEN (HEX) KEY 16MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER INTERNAL STRAIGHT 175MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER INTERNAL BENT 175MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL STRAIGHT 175MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL BENT 175MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER INTERNAL STRAIGHT 230MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIRCLIP PLIER EXTERNAL STRAIGHT 230MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHISEL SET (05 PCS SET)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIPE WRENCH SIZE 10"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIPE WRENCH SIZE 12"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIPE WRENCH SIZE 18"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIPE WRENCH SIZE 24"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIPE WRENCH SIZE 36"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLEDGE HAMMER 1 LBS WITH FIBREGLASS HANDLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SLEDGE HAMMER 3 LBS WITH FIBREGLASS HANDLE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOFT FACE DEAD BLOW HAMMER 50MM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VICE GRIP PLIER 08"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORDLESS IMPACT WRENCH 185NM (Bosch)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bosch Professional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORDLESS IMPACT WRENCH 350N (Bosch)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CORDLESS IMPACT WRENCH 1000N (Bosch)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HEX IMPACT ADAPTOR 1/2" FEMALE TO 1/4" FEMALE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DeWalt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FLAT FILE 12"</t>
-  </si>
-  <si>
     <t xml:space="preserve">ROUNDE FILE 12"</t>
   </si>
   <si>
@@ -280,72 +289,75 @@
     <t xml:space="preserve">CIRCUMFERENCE TAPE (60-950) (D20-300)</t>
   </si>
   <si>
+    <t xml:space="preserve">Insize / Equivalent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIRCUMFERENCE TAPE (940-2200) (D300-700)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEASURING TAPE 5M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS COBALT DRILL SET 1-13MM 25 PCS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BITS 1/16-1/2" 29 PCS SET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 14MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 15MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 15.5MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 16MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 16.5MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 17MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 17.5MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 19MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 21MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 25MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 30MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 32MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HSS DRILL BIT 35MM TAPER SHANK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEAD CENTRE DIAMOND TIP M2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEAD CENTRE DIAMOND TIP M3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIGITAL VERINER CALIPER 300MM (Insize brand)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Insize</t>
   </si>
   <si>
-    <t xml:space="preserve">CIRCUMFERENCE TAPE (940-2200) (D300-700)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEASURING TAPE 5M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS COBALT DRILL SET 1-13MM 25 PCS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BITS 1/16-1/2" 29 PCS SET</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 14MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 15MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 15.5MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 16MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 16.5MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 17MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 17.5MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 19MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 21MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 25MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 30MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 32MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HSS DRILL BIT 35MM TAPER SHANK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MORSE TAPER EXTENSION SOCKET SLEEVE ADAPT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEAD CENTRE DIAMOND TIP M2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEAD CENTRE DIAMOND TIP M3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIGITAL VERINER CALIPER 300MM (Insize brand)</t>
-  </si>
-  <si>
     <t xml:space="preserve">MANUAL VERNIER CALLIPER 12" (Insize brand)</t>
   </si>
   <si>
@@ -379,6 +391,9 @@
     <t xml:space="preserve">WELDING HELMET (FLIP FRONT)</t>
   </si>
   <si>
+    <t xml:space="preserve">Industrial / Equivalent</t>
+  </si>
+  <si>
     <t xml:space="preserve">WELDING LEATHER GLOVES 16"</t>
   </si>
   <si>
@@ -424,7 +439,7 @@
     <t xml:space="preserve">CYLINDER KEY/SPANNER</t>
   </si>
   <si>
-    <t xml:space="preserve">Draper</t>
+    <t xml:space="preserve">Draper / Equivalent</t>
   </si>
   <si>
     <t xml:space="preserve">TIP CLEANER FOR GAS WELDING TORCH</t>
@@ -1628,7 +1643,7 @@
         <v>34</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="D24" s="4" t="n">
         <v>3</v>
@@ -1646,10 +1661,10 @@
         <v>21</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D25" s="4" t="n">
         <v>3</v>
@@ -1667,10 +1682,10 @@
         <v>22</v>
       </c>
       <c r="B26" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>36</v>
       </c>
       <c r="D26" s="4" t="n">
         <v>3</v>
@@ -1688,7 +1703,7 @@
         <v>23</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>20</v>
@@ -1709,7 +1724,7 @@
         <v>24</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>20</v>
@@ -1730,7 +1745,7 @@
         <v>25</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>20</v>
@@ -1751,7 +1766,7 @@
         <v>26</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>20</v>
@@ -1772,7 +1787,7 @@
         <v>27</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>11</v>
@@ -1793,10 +1808,10 @@
         <v>28</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D32" s="4" t="n">
         <v>3</v>
@@ -1814,7 +1829,7 @@
         <v>30</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>20</v>
@@ -1835,10 +1850,10 @@
         <v>31</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D34" s="4" t="n">
         <v>3</v>
@@ -1856,7 +1871,7 @@
         <v>32</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>23</v>
@@ -1877,7 +1892,7 @@
         <v>33</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>20</v>
@@ -1898,7 +1913,7 @@
         <v>34</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>23</v>
@@ -1919,10 +1934,10 @@
         <v>35</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D38" s="4" t="n">
         <v>2</v>
@@ -1940,10 +1955,10 @@
         <v>36</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D39" s="4" t="n">
         <v>3</v>
@@ -1961,7 +1976,7 @@
         <v>37</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>23</v>
@@ -1982,7 +1997,7 @@
         <v>38</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>23</v>
@@ -2003,7 +2018,7 @@
         <v>39</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>20</v>
@@ -2024,10 +2039,10 @@
         <v>40</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D43" s="4" t="n">
         <v>3</v>
@@ -2045,10 +2060,10 @@
         <v>41</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D44" s="4" t="n">
         <v>3</v>
@@ -2066,10 +2081,10 @@
         <v>42</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D45" s="4" t="n">
         <v>2</v>
@@ -2087,10 +2102,10 @@
         <v>43</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D46" s="4" t="n">
         <v>4</v>
@@ -2108,10 +2123,10 @@
         <v>44</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="D47" s="4" t="n">
         <v>4</v>
@@ -2129,10 +2144,10 @@
         <v>45</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D48" s="4" t="n">
         <v>4</v>
@@ -2150,10 +2165,10 @@
         <v>47</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D49" s="4" t="n">
         <v>3</v>
@@ -2171,7 +2186,7 @@
         <v>48</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C50" s="4" t="s">
         <v>11</v>
@@ -2192,7 +2207,7 @@
         <v>49</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C51" s="4" t="s">
         <v>11</v>
@@ -2213,7 +2228,7 @@
         <v>50</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C52" s="4" t="s">
         <v>11</v>
@@ -2234,10 +2249,10 @@
         <v>51</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="D53" s="4" t="n">
         <v>1</v>
@@ -2255,10 +2270,10 @@
         <v>52</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="D54" s="4" t="n">
         <v>2</v>
@@ -2276,10 +2291,10 @@
         <v>53</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="D55" s="4" t="n">
         <v>1</v>
@@ -2297,10 +2312,10 @@
         <v>54</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D56" s="4" t="n">
         <v>2</v>
@@ -2318,7 +2333,7 @@
         <v>55</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C57" s="4" t="s">
         <v>11</v>
@@ -2339,10 +2354,10 @@
         <v>56</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D58" s="4" t="n">
         <v>1</v>
@@ -2360,7 +2375,7 @@
         <v>57</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C59" s="4" t="s">
         <v>20</v>
@@ -2381,7 +2396,7 @@
         <v>58</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C60" s="4" t="s">
         <v>11</v>
@@ -2402,7 +2417,7 @@
         <v>59</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C61" s="4" t="s">
         <v>11</v>
@@ -2423,10 +2438,10 @@
         <v>60</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D62" s="4" t="n">
         <v>2</v>
@@ -2444,10 +2459,10 @@
         <v>61</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C63" s="4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D63" s="4" t="n">
         <v>2</v>
@@ -2465,10 +2480,10 @@
         <v>62</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D64" s="4" t="n">
         <v>3</v>
@@ -2486,10 +2501,10 @@
         <v>63</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D65" s="4" t="n">
         <v>1</v>
@@ -2507,10 +2522,10 @@
         <v>64</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="D66" s="4" t="n">
         <v>3</v>
@@ -2528,10 +2543,10 @@
         <v>65</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="D67" s="4" t="n">
         <v>3</v>
@@ -2549,7 +2564,7 @@
         <v>66</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C68" s="4" t="s">
         <v>11</v>
@@ -2570,7 +2585,7 @@
         <v>67</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C69" s="4" t="s">
         <v>11</v>
@@ -2591,10 +2606,10 @@
         <v>69</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D70" s="4" t="n">
         <v>2</v>
@@ -2612,10 +2627,10 @@
         <v>70</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D71" s="4" t="n">
         <v>1</v>
@@ -2633,10 +2648,10 @@
         <v>71</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D72" s="4" t="n">
         <v>1</v>
@@ -2654,10 +2669,10 @@
         <v>73</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D73" s="4" t="n">
         <v>1</v>
@@ -2675,7 +2690,7 @@
         <v>74</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C74" s="4" t="s">
         <v>15</v>
@@ -2696,7 +2711,7 @@
         <v>75</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="C75" s="4" t="s">
         <v>15</v>
@@ -2717,7 +2732,7 @@
         <v>76</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C76" s="4" t="s">
         <v>15</v>
@@ -2738,7 +2753,7 @@
         <v>77</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C77" s="4" t="s">
         <v>15</v>
@@ -2759,7 +2774,7 @@
         <v>78</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C78" s="4" t="s">
         <v>15</v>
@@ -2780,7 +2795,7 @@
         <v>79</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C79" s="4" t="s">
         <v>15</v>
@@ -2801,7 +2816,7 @@
         <v>80</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C80" s="4" t="s">
         <v>15</v>
@@ -2822,7 +2837,7 @@
         <v>81</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C81" s="4" t="s">
         <v>15</v>
@@ -2843,7 +2858,7 @@
         <v>82</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C82" s="4" t="s">
         <v>15</v>
@@ -2864,7 +2879,7 @@
         <v>83</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C83" s="4" t="s">
         <v>15</v>
@@ -2885,7 +2900,7 @@
         <v>84</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C84" s="4" t="s">
         <v>15</v>
@@ -2906,7 +2921,7 @@
         <v>85</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C85" s="4" t="s">
         <v>15</v>
@@ -2927,7 +2942,7 @@
         <v>86</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C86" s="4" t="s">
         <v>15</v>
@@ -2948,7 +2963,7 @@
         <v>87</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C87" s="4" t="s">
         <v>15</v>
@@ -2969,7 +2984,7 @@
         <v>88</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C88" s="4" t="s">
         <v>11</v>
@@ -2990,7 +3005,7 @@
         <v>89</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>11</v>
@@ -3011,7 +3026,7 @@
         <v>90</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>11</v>
@@ -3032,7 +3047,7 @@
         <v>91</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C91" s="4" t="s">
         <v>11</v>
@@ -3053,7 +3068,7 @@
         <v>92</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C92" s="4" t="s">
         <v>11</v>
@@ -3074,10 +3089,10 @@
         <v>93</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="D93" s="4" t="n">
         <v>2</v>
@@ -3095,10 +3110,10 @@
         <v>94</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="D94" s="4" t="n">
         <v>3</v>
@@ -3116,10 +3131,10 @@
         <v>95</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="D95" s="4" t="n">
         <v>3</v>
@@ -3137,10 +3152,10 @@
         <v>96</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D96" s="4" t="n">
         <v>2</v>
@@ -3158,10 +3173,10 @@
         <v>97</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D97" s="4" t="n">
         <v>2</v>
@@ -3179,7 +3194,7 @@
         <v>98</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C98" s="4" t="s">
         <v>15</v>
@@ -3200,7 +3215,7 @@
         <v>99</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C99" s="4" t="s">
         <v>15</v>
@@ -3221,7 +3236,7 @@
         <v>100</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C100" s="4" t="s">
         <v>15</v>
@@ -3242,7 +3257,7 @@
         <v>101</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C101" s="4" t="s">
         <v>15</v>
@@ -3263,7 +3278,7 @@
         <v>102</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C102" s="4" t="s">
         <v>15</v>
@@ -3284,7 +3299,7 @@
         <v>103</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C103" s="4" t="s">
         <v>9</v>
@@ -3305,10 +3320,10 @@
         <v>104</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D104" s="4" t="n">
         <v>4</v>
@@ -3326,7 +3341,7 @@
         <v>105</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="C105" s="4" t="s">
         <v>9</v>
@@ -3347,10 +3362,10 @@
         <v>106</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D106" s="4" t="n">
         <v>6</v>
@@ -3368,10 +3383,10 @@
         <v>107</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D107" s="4" t="n">
         <v>6</v>
@@ -3389,10 +3404,10 @@
         <v>108</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D108" s="4" t="n">
         <v>3</v>
@@ -3410,10 +3425,10 @@
         <v>109</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D109" s="4" t="n">
         <v>6</v>
@@ -3431,10 +3446,10 @@
         <v>110</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D110" s="4" t="n">
         <v>3</v>
@@ -3452,7 +3467,7 @@
         <v>111</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C111" s="4" t="s">
         <v>23</v>
@@ -3473,7 +3488,7 @@
         <v>112</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C112" s="4" t="s">
         <v>9</v>
@@ -3494,7 +3509,7 @@
         <v>113</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C113" s="4" t="s">
         <v>9</v>
@@ -3515,7 +3530,7 @@
         <v>114</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C114" s="4" t="s">
         <v>9</v>
@@ -3536,7 +3551,7 @@
         <v>115</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C115" s="4" t="s">
         <v>9</v>
@@ -3557,10 +3572,10 @@
         <v>116</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D116" s="4" t="n">
         <v>2</v>
@@ -3578,10 +3593,10 @@
         <v>117</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D117" s="4" t="n">
         <v>15</v>
@@ -3599,10 +3614,10 @@
         <v>118</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D118" s="4" t="n">
         <v>15</v>
@@ -3620,10 +3635,10 @@
         <v>119</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D119" s="4" t="n">
         <v>2</v>
@@ -3641,10 +3656,10 @@
         <v>120</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D120" s="4" t="n">
         <v>6</v>
@@ -3662,7 +3677,7 @@
         <v>121</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C121" s="4" t="s">
         <v>9</v>
@@ -3683,7 +3698,7 @@
         <v>122</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="C122" s="4" t="s">
         <v>9</v>
@@ -3704,10 +3719,10 @@
         <v>123</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D123" s="4" t="n">
         <v>2</v>
@@ -3725,10 +3740,10 @@
         <v>124</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D124" s="4" t="n">
         <v>2</v>
@@ -3746,10 +3761,10 @@
         <v>125</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D125" s="4" t="n">
         <v>12</v>
@@ -3767,10 +3782,10 @@
         <v>126</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D126" s="4" t="n">
         <v>12</v>
@@ -3788,10 +3803,10 @@
         <v>127</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D127" s="4" t="n">
         <v>6</v>
@@ -3809,10 +3824,10 @@
         <v>128</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D128" s="4" t="n">
         <v>6</v>
@@ -3830,10 +3845,10 @@
         <v>129</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D129" s="4" t="n">
         <v>6</v>
@@ -3851,10 +3866,10 @@
         <v>130</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D130" s="4" t="n">
         <v>6</v>
@@ -3872,7 +3887,7 @@
         <v>131</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C131" s="4" t="s">
         <v>9</v>
@@ -3893,10 +3908,10 @@
         <v>132</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D132" s="4" t="n">
         <v>10</v>
@@ -3914,10 +3929,10 @@
         <v>133</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D133" s="4" t="n">
         <v>6</v>
@@ -3935,10 +3950,10 @@
         <v>134</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D134" s="4" t="n">
         <v>6</v>
@@ -3956,7 +3971,7 @@
         <v>135</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C135" s="4" t="s">
         <v>9</v>
@@ -3977,7 +3992,7 @@
         <v>136</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C136" s="4" t="s">
         <v>9</v>
@@ -3998,7 +4013,7 @@
         <v>138</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C137" s="4" t="s">
         <v>9</v>
@@ -4019,7 +4034,7 @@
         <v>139</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="C138" s="4" t="s">
         <v>11</v>
@@ -4040,10 +4055,10 @@
         <v>140</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D139" s="4" t="n">
         <v>24</v>
@@ -4061,10 +4076,10 @@
         <v>142</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D140" s="4" t="n">
         <v>3</v>
@@ -4082,10 +4097,10 @@
         <v>143</v>
       </c>
       <c r="B141" s="4" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C141" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D141" s="4" t="n">
         <v>3</v>
@@ -4103,10 +4118,10 @@
         <v>144</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D142" s="4" t="n">
         <v>3</v>
@@ -4124,7 +4139,7 @@
         <v>145</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C143" s="4" t="s">
         <v>11</v>
@@ -4145,7 +4160,7 @@
         <v>146</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C144" s="4" t="s">
         <v>9</v>
@@ -4166,7 +4181,7 @@
         <v>147</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C145" s="4" t="s">
         <v>9</v>
@@ -4187,7 +4202,7 @@
         <v>148</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C146" s="4" t="s">
         <v>27</v>
@@ -4208,10 +4223,10 @@
         <v>149</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="D147" s="4" t="n">
         <v>100</v>
@@ -4229,7 +4244,7 @@
         <v>150</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C148" s="4" t="s">
         <v>9</v>
@@ -4250,7 +4265,7 @@
         <v>151</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C149" s="4" t="s">
         <v>9</v>
@@ -4271,7 +4286,7 @@
         <v>152</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C150" s="4" t="s">
         <v>9</v>
@@ -4292,7 +4307,7 @@
         <v>153</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C151" s="4" t="s">
         <v>9</v>
@@ -4313,10 +4328,10 @@
         <v>154</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D152" s="4" t="n">
         <v>12</v>
@@ -4334,7 +4349,7 @@
         <v>155</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C153" s="4" t="s">
         <v>9</v>
@@ -4355,7 +4370,7 @@
         <v>156</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C154" s="4" t="s">
         <v>9</v>
@@ -4376,7 +4391,7 @@
         <v>157</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C155" s="4" t="s">
         <v>9</v>
@@ -4397,10 +4412,10 @@
         <v>158</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D156" s="4" t="n">
         <v>12</v>
@@ -4418,10 +4433,10 @@
         <v>159</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D157" s="4" t="n">
         <v>100</v>
@@ -4439,10 +4454,10 @@
         <v>160</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="D158" s="4" t="n">
         <v>150</v>
@@ -4460,7 +4475,7 @@
         <v>161</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C159" s="4" t="s">
         <v>11</v>
@@ -4481,7 +4496,7 @@
         <v>162</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C160" s="4" t="s">
         <v>11</v>
@@ -4502,7 +4517,7 @@
         <v>164</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C161" s="4" t="s">
         <v>9</v>
@@ -4523,7 +4538,7 @@
         <v>165</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C162" s="4" t="s">
         <v>9</v>
@@ -4544,7 +4559,7 @@
         <v>166</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="C163" s="4" t="s">
         <v>9</v>
@@ -4565,7 +4580,7 @@
         <v>167</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C164" s="4" t="s">
         <v>9</v>
@@ -4586,7 +4601,7 @@
         <v>168</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C165" s="4" t="s">
         <v>9</v>
@@ -4607,7 +4622,7 @@
         <v>177</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C166" s="4" t="s">
         <v>11</v>
@@ -4628,7 +4643,7 @@
         <v>179</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="C167" s="4" t="s">
         <v>15</v>
@@ -4649,7 +4664,7 @@
         <v>180</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C168" s="4" t="s">
         <v>15</v>
@@ -4670,7 +4685,7 @@
         <v>181</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="C169" s="4" t="s">
         <v>15</v>
@@ -4691,7 +4706,7 @@
         <v>182</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C170" s="4" t="s">
         <v>15</v>
@@ -4712,7 +4727,7 @@
         <v>183</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C171" s="4" t="s">
         <v>15</v>
@@ -4733,10 +4748,10 @@
         <v>184</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C172" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D172" s="4" t="n">
         <v>3</v>
@@ -4754,7 +4769,7 @@
         <v>185</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="C173" s="4" t="s">
         <v>15</v>
@@ -4775,10 +4790,10 @@
         <v>186</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C174" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D174" s="4" t="n">
         <v>3</v>
@@ -4796,10 +4811,10 @@
         <v>187</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="C175" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D175" s="4" t="n">
         <v>2</v>
@@ -4817,7 +4832,7 @@
         <v>188</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C176" s="4" t="s">
         <v>15</v>
@@ -4838,10 +4853,10 @@
         <v>189</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D177" s="4" t="n">
         <v>1</v>
@@ -4859,10 +4874,10 @@
         <v>190</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D178" s="4" t="n">
         <v>2</v>
@@ -4880,10 +4895,10 @@
         <v>191</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D179" s="4" t="n">
         <v>2</v>
@@ -4901,10 +4916,10 @@
         <v>192</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D180" s="4" t="n">
         <v>3</v>
@@ -4922,10 +4937,10 @@
         <v>193</v>
       </c>
       <c r="B181" s="4" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C181" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D181" s="4" t="n">
         <v>2</v>
@@ -4943,10 +4958,10 @@
         <v>194</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="C182" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D182" s="4" t="n">
         <v>3</v>
@@ -4964,10 +4979,10 @@
         <v>195</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="C183" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D183" s="4" t="n">
         <v>2</v>
@@ -4985,10 +5000,10 @@
         <v>196</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="C184" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D184" s="4" t="n">
         <v>2</v>
@@ -5006,10 +5021,10 @@
         <v>197</v>
       </c>
       <c r="B185" s="4" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="D185" s="4" t="n">
         <v>1</v>
@@ -5027,10 +5042,10 @@
         <v>198</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="C186" s="4" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="D186" s="4" t="n">
         <v>1</v>
@@ -5048,10 +5063,10 @@
         <v>199</v>
       </c>
       <c r="B187" s="4" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="D187" s="4" t="n">
         <v>1</v>
@@ -5069,10 +5084,10 @@
         <v>200</v>
       </c>
       <c r="B188" s="4" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="C188" s="4" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="D188" s="4" t="n">
         <v>1</v>
@@ -5090,10 +5105,10 @@
         <v>201</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="C189" s="4" t="s">
-        <v>86</v>
+        <v>111</v>
       </c>
       <c r="D189" s="4" t="n">
         <v>1</v>
@@ -5111,10 +5126,10 @@
         <v>202</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="C190" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D190" s="4" t="n">
         <v>2</v>
@@ -5132,7 +5147,7 @@
         <v>204</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C191" s="4" t="s">
         <v>15</v>
@@ -5153,7 +5168,7 @@
         <v>205</v>
       </c>
       <c r="B192" s="4" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="C192" s="4" t="s">
         <v>15</v>
@@ -5174,7 +5189,7 @@
         <v>206</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C193" s="4" t="s">
         <v>15</v>
@@ -5195,7 +5210,7 @@
         <v>207</v>
       </c>
       <c r="B194" s="4" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="C194" s="4" t="s">
         <v>15</v>
@@ -5216,10 +5231,10 @@
         <v>208</v>
       </c>
       <c r="B195" s="4" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C195" s="4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="D195" s="4" t="n">
         <v>3</v>
@@ -5237,7 +5252,7 @@
         <v>209</v>
       </c>
       <c r="B196" s="4" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="C196" s="4" t="s">
         <v>15</v>
@@ -5258,7 +5273,7 @@
         <v>210</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C197" s="4" t="s">
         <v>15</v>
@@ -5279,7 +5294,7 @@
         <v>211</v>
       </c>
       <c r="B198" s="4" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C198" s="4" t="s">
         <v>15</v>
@@ -5300,7 +5315,7 @@
         <v>212</v>
       </c>
       <c r="B199" s="4" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="C199" s="4" t="s">
         <v>15</v>
@@ -5321,10 +5336,10 @@
         <v>213</v>
       </c>
       <c r="B200" s="4" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D200" s="4" t="n">
         <v>2</v>
@@ -5342,10 +5357,10 @@
         <v>214</v>
       </c>
       <c r="B201" s="4" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D201" s="4" t="n">
         <v>2</v>
@@ -5363,10 +5378,10 @@
         <v>215</v>
       </c>
       <c r="B202" s="4" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="C202" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D202" s="4" t="n">
         <v>2</v>
@@ -5384,10 +5399,10 @@
         <v>216</v>
       </c>
       <c r="B203" s="4" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D203" s="4" t="n">
         <v>2</v>
@@ -5405,10 +5420,10 @@
         <v>217</v>
       </c>
       <c r="B204" s="4" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C204" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D204" s="4" t="n">
         <v>2</v>
@@ -5426,10 +5441,10 @@
         <v>218</v>
       </c>
       <c r="B205" s="4" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="C205" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D205" s="4" t="n">
         <v>2</v>
@@ -5447,10 +5462,10 @@
         <v>219</v>
       </c>
       <c r="B206" s="4" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="C206" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D206" s="4" t="n">
         <v>1</v>
@@ -5468,10 +5483,10 @@
         <v>220</v>
       </c>
       <c r="B207" s="4" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="C207" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D207" s="4" t="n">
         <v>1</v>
@@ -5489,10 +5504,10 @@
         <v>221</v>
       </c>
       <c r="B208" s="4" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="C208" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D208" s="4" t="n">
         <v>1</v>
@@ -5510,7 +5525,7 @@
         <v>222</v>
       </c>
       <c r="B209" s="4" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C209" s="4" t="s">
         <v>11</v>
@@ -5531,10 +5546,10 @@
         <v>223</v>
       </c>
       <c r="B210" s="4" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="C210" s="4" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D210" s="4" t="n">
         <v>2</v>
@@ -5552,7 +5567,7 @@
         <v>224</v>
       </c>
       <c r="B211" s="4" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="C211" s="4" t="s">
         <v>11</v>
@@ -5573,7 +5588,7 @@
         <v>225</v>
       </c>
       <c r="B212" s="4" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="C212" s="4" t="s">
         <v>11</v>
@@ -5594,7 +5609,7 @@
         <v>226</v>
       </c>
       <c r="B213" s="4" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="C213" s="4" t="s">
         <v>11</v>
@@ -5615,7 +5630,7 @@
         <v>227</v>
       </c>
       <c r="B214" s="4" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C214" s="4" t="s">
         <v>11</v>
@@ -5636,7 +5651,7 @@
         <v>228</v>
       </c>
       <c r="B215" s="4" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="C215" s="4" t="s">
         <v>11</v>
@@ -5657,7 +5672,7 @@
         <v>229</v>
       </c>
       <c r="B216" s="4" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="C216" s="4" t="s">
         <v>11</v>
@@ -5678,10 +5693,10 @@
         <v>230</v>
       </c>
       <c r="B217" s="4" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C217" s="4" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="D217" s="4" t="n">
         <v>1</v>
@@ -5699,10 +5714,10 @@
         <v>231</v>
       </c>
       <c r="B218" s="4" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="C218" s="4" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="D218" s="4" t="n">
         <v>1</v>
@@ -5720,10 +5735,10 @@
         <v>233</v>
       </c>
       <c r="B219" s="4" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="C219" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D219" s="4" t="n">
         <v>2</v>
@@ -5741,7 +5756,7 @@
         <v>234</v>
       </c>
       <c r="B220" s="4" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C220" s="4" t="s">
         <v>9</v>
@@ -5762,7 +5777,7 @@
         <v>235</v>
       </c>
       <c r="B221" s="4" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C221" s="4" t="s">
         <v>9</v>
@@ -5783,10 +5798,10 @@
         <v>236</v>
       </c>
       <c r="B222" s="4" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C222" s="4" t="s">
-        <v>9</v>
+        <v>123</v>
       </c>
       <c r="D222" s="4" t="n">
         <v>200</v>
@@ -5804,7 +5819,7 @@
         <v>237</v>
       </c>
       <c r="B223" s="4" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="C223" s="4" t="s">
         <v>9</v>
@@ -5825,10 +5840,10 @@
         <v>238</v>
       </c>
       <c r="B224" s="4" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="C224" s="4" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D224" s="4" t="n">
         <v>6</v>
@@ -5846,10 +5861,10 @@
         <v>239</v>
       </c>
       <c r="B225" s="4" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C225" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D225" s="4" t="n">
         <v>50</v>
@@ -5867,7 +5882,7 @@
         <v>240</v>
       </c>
       <c r="B226" s="4" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="C226" s="4" t="s">
         <v>15</v>
@@ -5885,7 +5900,7 @@
     </row>
     <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E227" s="6" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="F227" s="7" t="n">
         <f aca="false">SUM(F5:F226)</f>

</xml_diff>

<commit_message>
Fix Licota 7-drawer trolley selling rate at 270,000 (Hassan's override)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4c5Y1XBRj63SkdBZ73bUS
</commit_message>
<xml_diff>
--- a/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
+++ b/quotes/PR-217-228/Zidane_Revised_Quotation_PR217_PR228.xlsx
@@ -1397,11 +1397,11 @@
         <v>3</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>313310</v>
+        <v>270000</v>
       </c>
       <c r="F12" s="5" t="n">
         <f aca="false">D12*E12</f>
-        <v>939930</v>
+        <v>810000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="F227" s="7" t="n">
         <f aca="false">SUM(F5:F226)</f>
-        <v>15769745</v>
+        <v>15639815</v>
       </c>
     </row>
   </sheetData>

</xml_diff>